<commit_message>
feat(F-NAR-016): TREE-DIF-061 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-061.xlsx
+++ b/stories/arbres/TREE-DIF-061.xlsx
@@ -15083,12 +15083,12 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Le caillou reste sourd, sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis vent ! Aniss pointe la porte, du doigt. Le porche garde l'air, trop fermé. Tes yeux vont plus loin, Aniss. La marche du seuil est encore sèche. Un rai de soleil reste trop mince. Vous faites comment, tous les deux ?</t>
+          <t>Le caillou reste lourd, sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis vent ! Aniss pointe la porte, du doigt. Le porche garde l'air, trop fermé. Tes yeux vont plus loin, Aniss. La marche du seuil est encore sèche. Un rai de soleil reste trop mince. Vous faites comment, tous les deux ?</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Le caillou reste sourd, sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis vent ! Aniss pointe la porte, du doigt. Le porche garde l'air, trop fermé. Tes yeux vont plus loin, Aniss. La marche du seuil est encore sèche. Un rai de soleil reste trop mince. Vous faites comment, tous les deux ?</t>
+          <t>Le caillou reste lourd, sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis vent ! Aniss pointe la porte, du doigt. Le porche garde l'air, trop fermé. Tes yeux vont plus loin, Aniss. La marche du seuil est encore sèche. Un rai de soleil reste trop mince. Vous faites comment, tous les deux ?</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -15223,7 +15223,7 @@
       <c r="AV80" s="2" t="inlineStr"/>
       <c r="AW80" t="inlineStr">
         <is>
-          <t>narrateur|Le caillou reste sourd, sous le porche.
+          <t>narrateur|Le caillou reste lourd, sous le porche.
 copine|Ça ne tourne plus, Aniss !
 narrateur|Mila souffle trop vite, trop fort.
 copine|Dis vent !
@@ -16489,7 +16489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16532,6 +16532,20 @@
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-019): TREE-DIF-061 polish Le moulin de papier d'Aniss et la grille de l'école
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-061.xlsx
+++ b/stories/arbres/TREE-DIF-061.xlsx
@@ -1197,17 +1197,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un bus passe, trop large, le long du muret. Dans le sac d'Aniss, le papier répond, tout sec. Le bitume fume, un peu mouillé, sous les bottes. Une odeur de pain chaud remonte le muret. Le boulanger a ouvert, Aniss. La grille de l'école brille, un peu froide. Le porche garde son ombre, plus loin. Ton moulin dépasse du sac. Aniss sort le bâton, et la goutte de cire rouge. Cette goutte, tu l'as mise hier soir. Elle tient la pale, contre le vent. En ce moment, Aniss serre le bâton contre sa veste. Je le plante à la grille, avant le porche. Mila arrive, les bottes trop pressées. Mila arrive, tu lui montres ? Aniss hoche la tête, tout petit. Les bottes de Mila tapent le bitume, derrière. Dis tourne, Aniss ! Aniss lève le moulin trop vite, vers la grille. Le bâton bute contre deux barreaux, trop serrés. Il ne passe pas. Le sourire d'Aniss disparaît, un instant. Dans sa poitrine, l'envie et l'inquiétude se bousculent. On prépare, puis on pose. Papa s'accroupit, à la hauteur d'Aniss. Merci, tu as tendu le papier, sans crier. Le fil et le caillou voyagent aussi.</t>
+          <t>Un bus passe, trop large, le long du muret. Dans le sac d'Aniss, le papier répond, tout sec. Le bitume fume, un peu mouillé, sous les bottes. Une odeur de pain chaud remonte le muret. Le boulanger a ouvert, Aniss. La grille de l'école brille, un peu froide. Le porche garde son ombre, plus loin. Ton moulin dépasse du sac. Aniss sort le bâton, et la goutte de cire rouge. Cette goutte, tu l'as mise hier soir. Elle tient la pale, contre le vent. En ce moment, Aniss serre le bâton contre sa veste. Je le plante à la grille, avant le porche. Mila arrive, les bottes trop pressées. Tu lui montres le moulin ? Aniss hoche la tête, tout petit. Les bottes de Mila tapent le bitume, derrière. Dis tourne, Aniss ! Aniss lève le moulin trop vite, vers la grille. Le bâton bute contre deux barreaux, trop serrés. Il ne passe pas. Le sourire d'Aniss disparaît, un instant. Dans sa poitrine, l'envie et l'inquiétude se bousculent. On prépare, puis on pose. Papa s'accroupit, à la hauteur d'Aniss. Merci, tu as tendu le papier, sans crier. Le fil et le caillou voyagent aussi.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un bus passe, trop large, le long du muret. Dans le sac d'Aniss, le papier répond, tout sec. Le bitume fume, un peu mouillé, sous les bottes. Une odeur de pain chaud remonte le muret. Le boulanger a ouvert, Aniss. La grille de l'école brille, un peu froide. Le porche garde son ombre, plus loin. Ton moulin dépasse du sac. Aniss sort le bâton, et la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;. Cette goutte, tu l'as mise hier soir. Elle tient la pale, contre le vent. En ce moment, Aniss serre le bâton contre sa veste. Je le plante à la grille, avant le porche. Mila arrive, les bottes trop pressées. Mila arrive, tu lui montres ? Aniss hoche la tête, tout petit. Les bottes de Mila tapent le bitume, derrière. Dis tourne, Aniss ! Aniss lève le moulin trop vite, vers la grille. Le bâton bute contre deux barreaux, trop serrés. Il ne passe pas. Le sourire d'Aniss disparaît, un instant. Dans sa poitrine, l'envie et l'inquiétude se bousculent. On prépare, puis on pose. Papa s'accroupit, à la hauteur d'Aniss. Merci, tu as tendu le papier, sans crier. Le fil et le caillou voyagent aussi.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un bus passe, trop large, le long du muret. Dans le sac d'Aniss, le papier répond, tout sec. Le bitume fume, un peu mouillé, sous les bottes. Une odeur de pain chaud remonte le muret. Le boulanger a ouvert, Aniss. La grille de l'école brille, un peu froide. Le porche garde son ombre, plus loin. Ton moulin dépasse du sac. Aniss sort le bâton, et la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;. Cette goutte, tu l'as mise hier soir. Elle tient la pale, contre le vent. En ce moment, Aniss serre le bâton contre sa veste. Je le plante à la grille, avant le porche. Mila arrive, les bottes trop pressées. Tu lui montres le moulin ? Aniss hoche la tête, tout petit. Les bottes de Mila tapent le bitume, derrière. Dis tourne, Aniss ! Aniss lève le moulin trop vite, vers la grille. Le bâton bute contre deux barreaux, trop serrés. Il ne passe pas. Le sourire d'Aniss disparaît, un instant. Dans sa poitrine, l'envie et l'inquiétude se bousculent. On prépare, puis on pose. Papa s'accroupit, à la hauteur d'Aniss. Merci, tu as tendu le papier, sans crier. Le fil et le caillou voyagent aussi.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Un bus passe, trop large, le long du muret. Dans le sac d'Aniss, le papier répond, tout sec. Le bitume fume, un peu mouillé, sous les bottes. Une odeur de pain chaud remonte le muret. Le boulanger a ouvert, Aniss. La grille de l'école brille, un peu froide. Le porche garde son ombre, plus loin. Ton moulin dépasse du sac. Aniss sort le bâton, et la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;. Cette goutte, tu l'as mise hier soir. Elle tient la pale, contre le vent. En ce moment, Aniss serre le bâton contre sa veste. Je le plante à la grille, avant le porche. Mila arrive, les bottes trop pressées. Mila arrive, tu lui montres ? Aniss hoche la tête, tout petit. Les bottes de Mila tapent le bitume, derrière. Dis tourne, Aniss ! Aniss lève le moulin trop vite, vers la grille. Le bâton bute contre deux barreaux, trop serrés. Il ne passe pas. Le sourire d'Aniss disparaît, un instant. Dans sa poitrine, l'envie et l'inquiétude se bousculent. On prépare, puis on pose. Papa s'accroupit, à la hauteur d'Aniss. Merci, tu as tendu le papier, sans crier. Le fil et le caillou voyagent aussi. [pause]</t>
+          <t>Un bus passe, trop large, le long du muret. Dans le sac d'Aniss, le papier répond, tout sec. Le bitume fume, un peu mouillé, sous les bottes. Une odeur de pain chaud remonte le muret. Le boulanger a ouvert, Aniss. La grille de l'école brille, un peu froide. Le porche garde son ombre, plus loin. Ton moulin dépasse du sac. Aniss sort le bâton, et la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;. Cette goutte, tu l'as mise hier soir. Elle tient la pale, contre le vent. En ce moment, Aniss serre le bâton contre sa veste. Je le plante à la grille, avant le porche. Mila arrive, les bottes trop pressées. Tu lui montres le moulin ? Aniss hoche la tête, tout petit. Les bottes de Mila tapent le bitume, derrière. Dis tourne, Aniss ! Aniss lève le moulin trop vite, vers la grille. Le bâton bute contre deux barreaux, trop serrés. Il ne passe pas. Le sourire d'Aniss disparaît, un instant. Dans sa poitrine, l'envie et l'inquiétude se bousculent. On prépare, puis on pose. Papa s'accroupit, à la hauteur d'Aniss. Merci, tu as tendu le papier, sans crier. Le fil et le caillou voyagent aussi. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1355,7 +1355,7 @@
 narrateur|En ce moment, Aniss serre le bâton contre sa veste.
 enfant-m|Je le plante à la grille, avant le porche.
 narrateur|Mila arrive, les bottes trop pressées.
-papa|Mila arrive, tu lui montres ?
+papa|Tu lui montres le moulin ?
 narrateur|Aniss hoche la tête, tout petit.
 narrateur|Les bottes de Mila tapent le bitume, derrière.
 copine|Dis tourne, Aniss !
@@ -2354,17 +2354,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Le bâton du moulin bute contre deux barreaux. La grille serre trop, juste à hauteur d'Aniss. Pousse-le, Aniss ! Aniss montre un écart plus bas, du doigt. Le fer reste froid, trop près des pales. Dis-moi où ! Aniss secoue la tête, tout petit. On ne fonce pas. Mila se tait, et son silence compte. Il montre, avec le doigt. Le crochet du loquet brille un peu. La goutte de cire rouge s'est cachée derrière un barreau. Vous faites comment, tous les deux ?</t>
+          <t>Le bâton du moulin bute contre deux barreaux. La grille serre trop, juste à hauteur d'Aniss. Pousse-le, Aniss ! Aniss montre un écart plus bas, du doigt. Le fer reste froid, trop près des pales. Dis-moi où ! Aniss secoue la tête, tout petit. On ne fonce pas. Mila se tait, les mains ouvertes. Il montre, avec le doigt. Le crochet du loquet brille un peu. La goutte de cire rouge s'est cachée derrière un barreau. Vous faites comment, tous les deux ?</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le bâton du moulin bute contre deux barreaux. La grille serre trop, juste à hauteur d'Aniss. Pousse-le, Aniss ! Aniss montre un écart plus bas, du doigt. Le fer reste froid, trop près des pales. Dis-moi où ! Aniss secoue la tête, tout petit. On ne fonce pas. Mila se tait, et son silence compte. Il montre, avec le doigt. Le crochet du loquet brille un peu. La &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; s'est cachée derrière un barreau. Vous faites comment, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le bâton du moulin bute contre deux barreaux. La grille serre trop, juste à hauteur d'Aniss. Pousse-le, Aniss ! Aniss montre un écart plus bas, du doigt. Le fer reste froid, trop près des pales. Dis-moi où ! Aniss secoue la tête, tout petit. On ne fonce pas. Mila se tait, les mains ouvertes. Il montre, avec le doigt. Le crochet du loquet brille un peu. La &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; s'est cachée derrière un barreau. Vous faites comment, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Le bâton du moulin bute contre deux barreaux. La grille serre trop, juste à hauteur d'Aniss. Pousse-le, Aniss ! Aniss montre un écart plus bas, du doigt. Le fer reste froid, trop près des pales. Dis-moi où ! Aniss secoue la tête, tout petit. On ne fonce pas. Mila se tait, et son silence compte. Il montre, avec le doigt. Le crochet du loquet brille un peu. La &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; s'est cachée derrière un barreau. Vous faites comment, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Le bâton du moulin bute contre deux barreaux. La grille serre trop, juste à hauteur d'Aniss. Pousse-le, Aniss ! Aniss montre un écart plus bas, du doigt. Le fer reste froid, trop près des pales. Dis-moi où ! Aniss secoue la tête, tout petit. On ne fonce pas. Mila se tait, les mains ouvertes. Il montre, avec le doigt. Le crochet du loquet brille un peu. La &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; s'est cachée derrière un barreau. Vous faites comment, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -2510,7 +2510,7 @@
 copine|Dis-moi où !
 narrateur|Aniss secoue la tête, tout petit.
 enfant-m|On ne fonce pas.
-narrateur|Mila se tait, et son silence compte.
+narrateur|Mila se tait, les mains ouvertes.
 maman|Il montre, avec le doigt.
 papa|Le crochet du loquet brille un peu.
 narrateur|La goutte de cire rouge s'est cachée derrière un barreau.
@@ -2743,17 +2743,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>On attend. Aniss cherche l'écart du bas, sans presser. Mila suit le doigt, enfin, un peu. Le moulin reste bas, près du bitume. Aniss glisse le bâton, sans un mot. Le fer fait toc, plus large. Toc. La goutte de cire rouge revoit le vent, ronde. Le moulin attend, collé aux doigts. Le bas laisse un vrai passage. Il tourne.</t>
+          <t>On attend. Aniss cherche l'écart du bas, sans presser. Mila suit le doigt, enfin, un peu. Le moulin reste bas, près du bitume. Aniss glisse le bâton, sans un mot. Le fer fait toc, plus large. Toc. La goutte de cire rouge revoit le vent, ronde. Le moulin attend, collé aux doigts. Le bas laisse un vrai passage. En bas.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend. Aniss cherche l'écart du &lt;emphasis level="moderate"&gt;bas&lt;/emphasis&gt;, sans presser. Mila suit le doigt, enfin, un peu. Le moulin reste bas, près du bitume. Aniss glisse le bâton, sans un mot. Le fer fait toc, plus large. Toc. La goutte de cire rouge revoit le vent, ronde. Le moulin attend, collé aux doigts. Le bas laisse un vrai passage. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend. Aniss cherche l'écart du &lt;emphasis level="moderate"&gt;bas&lt;/emphasis&gt;, sans presser. Mila suit le doigt, enfin, un peu. Le moulin reste bas, près du bitume. Aniss glisse le bâton, sans un mot. Le fer fait toc, plus large. Toc. La goutte de cire rouge revoit le vent, ronde. Le moulin attend, collé aux doigts. Le bas laisse un vrai passage. En bas.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>On attend. Aniss cherche l'écart du &lt;emphasis&gt;bas&lt;/emphasis&gt;, sans presser. Mila suit le doigt, enfin, un peu. Le moulin reste bas, près du bitume. Aniss glisse le bâton, sans un mot. Le fer fait toc, plus large. Toc. La goutte de cire rouge revoit le vent, ronde. Le moulin attend, collé aux doigts. Le bas laisse un vrai passage. Il tourne. [pause]</t>
+          <t>On attend. Aniss cherche l'écart du &lt;emphasis&gt;bas&lt;/emphasis&gt;, sans presser. Mila suit le doigt, enfin, un peu. Le moulin reste bas, près du bitume. Aniss glisse le bâton, sans un mot. Le fer fait toc, plus large. Toc. La goutte de cire rouge revoit le vent, ronde. Le moulin attend, collé aux doigts. Le bas laisse un vrai passage. En bas. [pause]</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -2897,7 +2897,7 @@
 narrateur|La goutte de cire rouge revoit le vent, ronde.
 narrateur|Le moulin attend, collé aux doigts.
 papa|Le bas laisse un vrai passage.
-enfant-m|Il tourne.</t>
+enfant-m|En bas.</t>
         </is>
       </c>
       <c r="AX10" t="inlineStr">
@@ -3116,17 +3116,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Pour toi. Mila ouvre les deux mains, tout près. Aniss pose le jaune contre ses paumes. Le moulin glisse vers les mains de Mila. Mila vise l'écart, Aniss pousse le bâton. Il passe ! La goutte de cire rouge échappe au fer, ronde. Le moulin attend, collé aux doigts. Tes mains ont trouvé le fer. Il l'a tendu, d'abord. Il tourne.</t>
+          <t>Pour toi. Mila ouvre les deux mains, tout près. Aniss pose le jaune contre ses paumes. Le moulin glisse vers les mains de Mila. Mila vise l'écart, Aniss pousse le bâton. Il passe ! La goutte de cire rouge échappe au fer, ronde. Le moulin attend, collé aux doigts. Tes mains ont trouvé le fer. Il l'a tendu, d'abord. Tes mains.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Pour toi. Mila ouvre les deux &lt;emphasis level="moderate"&gt;mains&lt;/emphasis&gt;, tout près. Aniss pose le jaune contre ses paumes. Le moulin glisse vers les mains de Mila. Mila vise l'écart, Aniss pousse le bâton. Il passe ! La goutte de cire rouge échappe au fer, ronde. Le moulin attend, collé aux doigts. Tes mains ont trouvé le fer. Il l'a tendu, d'abord. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Pour toi. Mila ouvre les deux &lt;emphasis level="moderate"&gt;mains&lt;/emphasis&gt;, tout près. Aniss pose le jaune contre ses paumes. Le moulin glisse vers les mains de Mila. Mila vise l'écart, Aniss pousse le bâton. Il passe ! La goutte de cire rouge échappe au fer, ronde. Le moulin attend, collé aux doigts. Tes mains ont trouvé le fer. Il l'a tendu, d'abord. Tes mains.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Pour toi. Mila ouvre les deux &lt;emphasis&gt;mains&lt;/emphasis&gt;, tout près. Aniss pose le jaune contre ses paumes. Le moulin glisse vers les mains de Mila. Mila vise l'écart, Aniss pousse le bâton. Il passe ! La goutte de cire rouge échappe au fer, ronde. Le moulin attend, collé aux doigts. Tes mains ont trouvé le fer. Il l'a tendu, d'abord. Il tourne. [pause]</t>
+          <t>Pour toi. Mila ouvre les deux &lt;emphasis&gt;mains&lt;/emphasis&gt;, tout près. Aniss pose le jaune contre ses paumes. Le moulin glisse vers les mains de Mila. Mila vise l'écart, Aniss pousse le bâton. Il passe ! La goutte de cire rouge échappe au fer, ronde. Le moulin attend, collé aux doigts. Tes mains ont trouvé le fer. Il l'a tendu, d'abord. Tes mains. [pause]</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -3270,7 +3270,7 @@
 narrateur|Le moulin attend, collé aux doigts.
 maman|Tes mains ont trouvé le fer.
 papa|Il l'a tendu, d'abord.
-enfant-m|Il tourne.</t>
+enfant-m|Tes mains.</t>
         </is>
       </c>
       <c r="AX12" t="inlineStr">
@@ -3489,17 +3489,17 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Le crochet, Aniss. Aniss lève le jaune, sans un mot. Mila attend, puis suit sa main. Le moulin pend au crochet du loquet. Une pale racle le fer, puis se libère. Il tient. La goutte de cire rouge reprend le rai, petite. Le moulin attend, collé aux doigts. Le loquet a gardé le papier. Les barreaux peuvent dormir, plus loin. Il tourne.</t>
+          <t>Le crochet, Aniss. Aniss lève le jaune, sans un mot. Mila attend, puis suit sa main. Le moulin pend au crochet du loquet. Une pale racle le fer, puis se libère. Il tient. La goutte de cire rouge reprend le rai, petite. Le moulin attend, collé aux doigts. Le loquet a gardé le papier. Les barreaux peuvent dormir, plus loin. Au crochet.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;crochet&lt;/emphasis&gt;, Aniss. Aniss lève le jaune, sans un mot. Mila attend, puis suit sa main. Le moulin pend au crochet du loquet. Une pale racle le fer, puis se libère. Il tient. La goutte de cire rouge reprend le rai, petite. Le moulin attend, collé aux doigts. Le loquet a gardé le papier. Les barreaux peuvent dormir, plus loin. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;crochet&lt;/emphasis&gt;, Aniss. Aniss lève le jaune, sans un mot. Mila attend, puis suit sa main. Le moulin pend au crochet du loquet. Une pale racle le fer, puis se libère. Il tient. La goutte de cire rouge reprend le rai, petite. Le moulin attend, collé aux doigts. Le loquet a gardé le papier. Les barreaux peuvent dormir, plus loin. Au crochet.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;crochet&lt;/emphasis&gt;, Aniss. Aniss lève le jaune, sans un mot. Mila attend, puis suit sa main. Le moulin pend au crochet du loquet. Une pale racle le fer, puis se libère. Il tient. La goutte de cire rouge reprend le rai, petite. Le moulin attend, collé aux doigts. Le loquet a gardé le papier. Les barreaux peuvent dormir, plus loin. Il tourne. [pause]</t>
+          <t>Le &lt;emphasis&gt;crochet&lt;/emphasis&gt;, Aniss. Aniss lève le jaune, sans un mot. Mila attend, puis suit sa main. Le moulin pend au crochet du loquet. Une pale racle le fer, puis se libère. Il tient. La goutte de cire rouge reprend le rai, petite. Le moulin attend, collé aux doigts. Le loquet a gardé le papier. Les barreaux peuvent dormir, plus loin. Au crochet. [pause]</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -3643,7 +3643,7 @@
 narrateur|Le moulin attend, collé aux doigts.
 papa|Le loquet a gardé le papier.
 maman|Les barreaux peuvent dormir, plus loin.
-enfant-m|Il tourne.</t>
+enfant-m|Au crochet.</t>
         </is>
       </c>
       <c r="AX14" t="inlineStr">
@@ -3862,17 +3862,17 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Une pale du moulin touche l'eau, trop vite. L'eau est trop grande. Une feuille jaune part, plus bas. Attrape, Aniss ! Aniss recule le papier, sans presser. L'eau frappe la dalle, puis rebondit. On ne fonce pas. Mila referme la bouche. Son silence compte, comme une réponse. La dalle tient le courant. On reste près du caniveau, tous les deux. La goutte de cire rouge s'est ternie, trop près de l'eau. Vous faites comment, tous les deux ?</t>
+          <t>Une pale du moulin touche l'eau, trop vite. L'eau est trop grande. Une feuille jaune part, plus bas. Attrape, Aniss ! Aniss recule le papier, sans presser. L'eau frappe la dalle, puis rebondit. Attends. Mila referme la bouche. Elle pose les mains, ouvertes, près du papier. La dalle tient le courant. On reste près du caniveau, tous les deux. La goutte de cire rouge s'est ternie, trop près de l'eau. Vous faites comment, tous les deux ?</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Une pale du moulin touche l'eau, trop vite. L'eau est trop grande. Une feuille jaune part, plus bas. Attrape, Aniss ! Aniss recule le papier, sans presser. L'eau frappe la dalle, puis rebondit. On ne fonce pas. Mila referme la bouche. Son silence compte, comme une réponse. La dalle tient le courant. On reste près du caniveau, tous les deux. La &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; s'est ternie, trop près de l'eau. Vous faites comment, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Une pale du moulin touche l'eau, trop vite. L'eau est trop grande. Une feuille jaune part, plus bas. Attrape, Aniss ! Aniss recule le papier, sans presser. L'eau frappe la dalle, puis rebondit. Attends. Mila referme la bouche. Elle pose les mains, ouvertes, près du papier. La dalle tient le courant. On reste près du caniveau, tous les deux. La &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; s'est ternie, trop près de l'eau. Vous faites comment, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Une pale du moulin touche l'eau, trop vite. L'eau est trop grande. Une feuille jaune part, plus bas. Attrape, Aniss ! Aniss recule le papier, sans presser. L'eau frappe la dalle, puis rebondit. On ne fonce pas. Mila referme la bouche. Son silence compte, comme une réponse. La dalle tient le courant. On reste près du caniveau, tous les deux. La &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; s'est ternie, trop près de l'eau. Vous faites comment, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Une pale du moulin touche l'eau, trop vite. L'eau est trop grande. Une feuille jaune part, plus bas. Attrape, Aniss ! Aniss recule le papier, sans presser. L'eau frappe la dalle, puis rebondit. Attends. Mila referme la bouche. Elle pose les mains, ouvertes, près du papier. La dalle tient le courant. On reste près du caniveau, tous les deux. La &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; s'est ternie, trop près de l'eau. Vous faites comment, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -4016,9 +4016,9 @@
 copine|Attrape, Aniss !
 narrateur|Aniss recule le papier, sans presser.
 narrateur|L'eau frappe la dalle, puis rebondit.
-enfant-m|On ne fonce pas.
+enfant-m|Attends.
 narrateur|Mila referme la bouche.
-narrateur|Son silence compte, comme une réponse.
+narrateur|Elle pose les mains, ouvertes, près du papier.
 maman|La dalle tient le courant.
 papa|On reste près du caniveau, tous les deux.
 narrateur|La goutte de cire rouge s'est ternie, trop près de l'eau.
@@ -4251,17 +4251,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>On attend l'eau. Aniss s'assoit près du caniveau, sans presser. Mila s'assoit aussi, les genoux contre lui. Le moulin sèche contre la dalle. L'eau frappe, puis la feuille s'arrête. Maintenant. La goutte de cire rouge sèche, ronde, sur la dalle. Le moulin attend, collé aux doigts. La dalle a cassé le courant. Vous avez laissé l'eau finir. Il tourne.</t>
+          <t>On attend l'eau. Aniss s'assoit près du caniveau, sans presser. Mila s'assoit aussi, les genoux contre lui. Le moulin sèche contre la dalle. L'eau frappe, puis la feuille s'arrête. Maintenant. La goutte de cire rouge sèche, ronde, sur la dalle. Le moulin attend, collé aux doigts. La dalle a cassé le courant. Vous avez laissé l'eau finir. La dalle.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend l'eau. Aniss s'assoit près du caniveau, sans presser. Mila s'assoit aussi, les genoux contre lui. Le moulin sèche contre la &lt;emphasis level="moderate"&gt;dalle&lt;/emphasis&gt;. L'eau frappe, puis la feuille s'arrête. Maintenant. La goutte de cire rouge sèche, ronde, sur la dalle. Le moulin attend, collé aux doigts. La dalle a cassé le courant. Vous avez laissé l'eau finir. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend l'eau. Aniss s'assoit près du caniveau, sans presser. Mila s'assoit aussi, les genoux contre lui. Le moulin sèche contre la &lt;emphasis level="moderate"&gt;dalle&lt;/emphasis&gt;. L'eau frappe, puis la feuille s'arrête. Maintenant. La goutte de cire rouge sèche, ronde, sur la dalle. Le moulin attend, collé aux doigts. La dalle a cassé le courant. Vous avez laissé l'eau finir. La dalle.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>On attend l'eau. Aniss s'assoit près du caniveau, sans presser. Mila s'assoit aussi, les genoux contre lui. Le moulin sèche contre la &lt;emphasis&gt;dalle&lt;/emphasis&gt;. L'eau frappe, puis la feuille s'arrête. Maintenant. La goutte de cire rouge sèche, ronde, sur la dalle. Le moulin attend, collé aux doigts. La dalle a cassé le courant. Vous avez laissé l'eau finir. Il tourne. [pause]</t>
+          <t>On attend l'eau. Aniss s'assoit près du caniveau, sans presser. Mila s'assoit aussi, les genoux contre lui. Le moulin sèche contre la &lt;emphasis&gt;dalle&lt;/emphasis&gt;. L'eau frappe, puis la feuille s'arrête. Maintenant. La goutte de cire rouge sèche, ronde, sur la dalle. Le moulin attend, collé aux doigts. La dalle a cassé le courant. Vous avez laissé l'eau finir. La dalle. [pause]</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -4405,7 +4405,7 @@
 narrateur|Le moulin attend, collé aux doigts.
 papa|La dalle a cassé le courant.
 maman|Vous avez laissé l'eau finir.
-enfant-m|Il tourne.</t>
+enfant-m|La dalle.</t>
         </is>
       </c>
       <c r="AX18" t="inlineStr">
@@ -4624,17 +4624,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Tes mains, Aniss. Aniss tend le fil, tout près. Mila tire avec lui, sans presser. Le moulin traverse au bout du fil. Le papier passe au-dessus de l'eau. On tient ensemble. La goutte de cire rouge tremble au bout du fil. Le moulin attend, collé aux doigts. Vos mains suffisent, toutes les deux. L'eau restera après. Il tourne.</t>
+          <t>Tes mains, Aniss. Aniss tend le fil, tout près. Mila tire avec lui, sans presser. Le moulin traverse au bout du fil. Le papier passe au-dessus de l'eau. On tient ensemble. La goutte de cire rouge tremble au bout du fil. Le moulin attend, collé aux doigts. Vos mains suffisent, toutes les deux. L'eau restera après. On tient.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tes mains, Aniss. Aniss tend le &lt;emphasis level="moderate"&gt;fil&lt;/emphasis&gt;, tout près. Mila tire avec lui, sans presser. Le moulin traverse au bout du fil. Le papier passe au-dessus de l'eau. On tient ensemble. La goutte de cire rouge tremble au bout du fil. Le moulin attend, collé aux doigts. Vos mains suffisent, toutes les deux. L'eau restera après. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tes mains, Aniss. Aniss tend le &lt;emphasis level="moderate"&gt;fil&lt;/emphasis&gt;, tout près. Mila tire avec lui, sans presser. Le moulin traverse au bout du fil. Le papier passe au-dessus de l'eau. On tient ensemble. La goutte de cire rouge tremble au bout du fil. Le moulin attend, collé aux doigts. Vos mains suffisent, toutes les deux. L'eau restera après. On tient.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Tes mains, Aniss. Aniss tend le &lt;emphasis&gt;fil&lt;/emphasis&gt;, tout près. Mila tire avec lui, sans presser. Le moulin traverse au bout du fil. Le papier passe au-dessus de l'eau. On tient ensemble. La goutte de cire rouge tremble au bout du fil. Le moulin attend, collé aux doigts. Vos mains suffisent, toutes les deux. L'eau restera après. Il tourne. [pause]</t>
+          <t>Tes mains, Aniss. Aniss tend le &lt;emphasis&gt;fil&lt;/emphasis&gt;, tout près. Mila tire avec lui, sans presser. Le moulin traverse au bout du fil. Le papier passe au-dessus de l'eau. On tient ensemble. La goutte de cire rouge tremble au bout du fil. Le moulin attend, collé aux doigts. Vos mains suffisent, toutes les deux. L'eau restera après. On tient. [pause]</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -4778,7 +4778,7 @@
 narrateur|Le moulin attend, collé aux doigts.
 maman|Vos mains suffisent, toutes les deux.
 papa|L'eau restera après.
-enfant-m|Il tourne.</t>
+enfant-m|On tient.</t>
         </is>
       </c>
       <c r="AX20" t="inlineStr">
@@ -4997,17 +4997,17 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Le bord, d'abord. Mila tend la pierre sèche vers Aniss. Aniss marche, sans un mot. Le moulin suit le bord sec. Une goutte rejoint le fond, puis se tait. C'est doux. La goutte de cire rouge reste au sec, sur le bord. Le moulin attend, collé aux doigts. L'eau garde son souffle, plus loin. Le bord a laissé le papier. Il tourne.</t>
+          <t>Le bord, d'abord. Mila tend la pierre sèche vers Aniss. Aniss marche, sans un mot. Le moulin suit le bord sec. Une goutte rejoint le fond, puis se tait. C'est doux. La goutte de cire rouge reste au sec, sur le bord. Le moulin attend, collé aux doigts. L'eau garde son souffle, plus loin. Le bord a laissé le papier. Au sec.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;bord&lt;/emphasis&gt;, d'abord. Mila tend la pierre sèche vers Aniss. Aniss marche, sans un mot. Le moulin suit le bord sec. Une goutte rejoint le fond, puis se tait. C'est doux. La goutte de cire rouge reste au sec, sur le bord. Le moulin attend, collé aux doigts. L'eau garde son souffle, plus loin. Le bord a laissé le papier. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;bord&lt;/emphasis&gt;, d'abord. Mila tend la pierre sèche vers Aniss. Aniss marche, sans un mot. Le moulin suit le bord sec. Une goutte rejoint le fond, puis se tait. C'est doux. La goutte de cire rouge reste au sec, sur le bord. Le moulin attend, collé aux doigts. L'eau garde son souffle, plus loin. Le bord a laissé le papier. Au sec.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;bord&lt;/emphasis&gt;, d'abord. Mila tend la pierre sèche vers Aniss. Aniss marche, sans un mot. Le moulin suit le bord sec. Une goutte rejoint le fond, puis se tait. C'est doux. La goutte de cire rouge reste au sec, sur le bord. Le moulin attend, collé aux doigts. L'eau garde son souffle, plus loin. Le bord a laissé le papier. Il tourne. [pause]</t>
+          <t>Le &lt;emphasis&gt;bord&lt;/emphasis&gt;, d'abord. Mila tend la pierre sèche vers Aniss. Aniss marche, sans un mot. Le moulin suit le bord sec. Une goutte rejoint le fond, puis se tait. C'est doux. La goutte de cire rouge reste au sec, sur le bord. Le moulin attend, collé aux doigts. L'eau garde son souffle, plus loin. Le bord a laissé le papier. Au sec. [pause]</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -5151,7 +5151,7 @@
 narrateur|Le moulin attend, collé aux doigts.
 maman|L'eau garde son souffle, plus loin.
 papa|Le bord a laissé le papier.
-enfant-m|Il tourne.</t>
+enfant-m|Au sec.</t>
         </is>
       </c>
       <c r="AX22" t="inlineStr">
@@ -5370,17 +5370,17 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Les pales du moulin s'arrêtent sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis vent ! Aniss pointe la porte, du doigt. Le porche garde l'air, trop fermé. On ne fonce pas. Mila se tait, les joues gonflées. Son silence compte, comme une réponse. Tes yeux vont plus loin, Aniss. La marche du seuil est sèche. La goutte de cire rouge s'est éteinte, dans l'ombre. Vous faites comment, tous les deux ?</t>
+          <t>Les pales du moulin s'arrêtent sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis vent ! Aniss pointe la porte, du doigt. Le porche garde l'air, trop fermé. Pas trop fort. Mila se tait, les joues gonflées. Elle pose les mains, ouvertes, sous le porche. Tes yeux vont plus loin, Aniss. La marche du seuil est sèche. La goutte de cire rouge s'est éteinte, dans l'ombre. Vous faites comment, tous les deux ?</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Les pales du moulin s'arrêtent sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis vent ! Aniss pointe la porte, du doigt. Le porche garde l'air, trop fermé. On ne fonce pas. Mila se tait, les joues gonflées. Son silence compte, comme une réponse. Tes yeux vont plus loin, Aniss. La marche du seuil est sèche. La &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; s'est éteinte, dans l'ombre. Vous faites comment, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Les pales du moulin s'arrêtent sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis vent ! Aniss pointe la porte, du doigt. Le porche garde l'air, trop fermé. Pas trop fort. Mila se tait, les joues gonflées. Elle pose les mains, ouvertes, sous le porche. Tes yeux vont plus loin, Aniss. La marche du seuil est sèche. La &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; s'est éteinte, dans l'ombre. Vous faites comment, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Les pales du moulin s'arrêtent sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis vent ! Aniss pointe la porte, du doigt. Le porche garde l'air, trop fermé. On ne fonce pas. Mila se tait, les joues gonflées. Son silence compte, comme une réponse. Tes yeux vont plus loin, Aniss. La marche du seuil est sèche. La &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; s'est éteinte, dans l'ombre. Vous faites comment, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Les pales du moulin s'arrêtent sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis vent ! Aniss pointe la porte, du doigt. Le porche garde l'air, trop fermé. Pas trop fort. Mila se tait, les joues gonflées. Elle pose les mains, ouvertes, sous le porche. Tes yeux vont plus loin, Aniss. La marche du seuil est sèche. La &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; s'est éteinte, dans l'ombre. Vous faites comment, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -5524,9 +5524,9 @@
 copine|Dis vent !
 narrateur|Aniss pointe la porte, du doigt.
 narrateur|Le porche garde l'air, trop fermé.
-enfant-m|On ne fonce pas.
+enfant-m|Pas trop fort.
 narrateur|Mila se tait, les joues gonflées.
-narrateur|Son silence compte, comme une réponse.
+narrateur|Elle pose les mains, ouvertes, sous le porche.
 maman|Tes yeux vont plus loin, Aniss.
 papa|La marche du seuil est sèche.
 narrateur|La goutte de cire rouge s'est éteinte, dans l'ombre.
@@ -5759,17 +5759,17 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Le vent, d'abord. J'ouvre un peu, à votre hauteur. Aniss attend, Mila tient le jaune. Le moulin prend le vent de la porte. Une pale part, sans un mot. Ça tient ! La goutte de cire rouge file dans le courant, ronde. Le moulin attend, collé aux doigts. La porte a donné le courant. Aniss a poussé, sans crier. Il tourne.</t>
+          <t>Le vent, d'abord. J'ouvre un peu, à votre hauteur. Aniss attend, Mila tient le jaune. Le moulin prend le vent de la porte. Une pale part, sans un mot. Ça tient ! La goutte de cire rouge file dans le courant, ronde. Le moulin attend, collé aux doigts. La porte a donné le courant. Aniss a poussé, sans crier. Le vent.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;vent&lt;/emphasis&gt;, d'abord. J'ouvre un peu, à votre hauteur. Aniss attend, Mila tient le jaune. Le moulin prend le vent de la porte. Une pale part, sans un mot. Ça tient ! La goutte de cire rouge file dans le courant, ronde. Le moulin attend, collé aux doigts. La porte a donné le courant. Aniss a poussé, sans crier. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;vent&lt;/emphasis&gt;, d'abord. J'ouvre un peu, à votre hauteur. Aniss attend, Mila tient le jaune. Le moulin prend le vent de la porte. Une pale part, sans un mot. Ça tient ! La goutte de cire rouge file dans le courant, ronde. Le moulin attend, collé aux doigts. La porte a donné le courant. Aniss a poussé, sans crier. Le vent.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;vent&lt;/emphasis&gt;, d'abord. J'ouvre un peu, à votre hauteur. Aniss attend, Mila tient le jaune. Le moulin prend le vent de la porte. Une pale part, sans un mot. Ça tient ! La goutte de cire rouge file dans le courant, ronde. Le moulin attend, collé aux doigts. La porte a donné le courant. Aniss a poussé, sans crier. Il tourne. [pause]</t>
+          <t>Le &lt;emphasis&gt;vent&lt;/emphasis&gt;, d'abord. J'ouvre un peu, à votre hauteur. Aniss attend, Mila tient le jaune. Le moulin prend le vent de la porte. Une pale part, sans un mot. Ça tient ! La goutte de cire rouge file dans le courant, ronde. Le moulin attend, collé aux doigts. La porte a donné le courant. Aniss a poussé, sans crier. Le vent. [pause]</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -5913,7 +5913,7 @@
 narrateur|Le moulin attend, collé aux doigts.
 papa|La porte a donné le courant.
 maman|Aniss a poussé, sans crier.
-enfant-m|Il tourne.</t>
+enfant-m|Le vent.</t>
         </is>
       </c>
       <c r="AX26" t="inlineStr">
@@ -6132,17 +6132,17 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Mila. Aniss pointe la marche, du doigt. Mila attend, puis ouvre les mains. Le moulin pose ses pales sur la marche. Le courant du seuil pousse, tout net. Je le tiens. La goutte de cire rouge prend l'air, sur la marche. Le moulin attend, collé aux doigts. Le porche garde son ombre, plus loin. Tes mains ont guidé le moulin. Il tourne.</t>
+          <t>Mila. Aniss pointe la marche, du doigt. Mila attend, puis ouvre les mains. Le moulin pose ses pales sur la marche. Le courant du seuil pousse, tout net. Je le tiens. La goutte de cire rouge prend l'air, sur la marche. Le moulin attend, collé aux doigts. Le porche garde son ombre, plus loin. Tes mains ont guidé le moulin. La marche.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila. Aniss pointe la &lt;emphasis level="moderate"&gt;marche&lt;/emphasis&gt;, du doigt. Mila attend, puis ouvre les mains. Le moulin pose ses pales sur la marche. Le courant du seuil pousse, tout net. Je le tiens. La goutte de cire rouge prend l'air, sur la marche. Le moulin attend, collé aux doigts. Le porche garde son ombre, plus loin. Tes mains ont guidé le moulin. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila. Aniss pointe la &lt;emphasis level="moderate"&gt;marche&lt;/emphasis&gt;, du doigt. Mila attend, puis ouvre les mains. Le moulin pose ses pales sur la marche. Le courant du seuil pousse, tout net. Je le tiens. La goutte de cire rouge prend l'air, sur la marche. Le moulin attend, collé aux doigts. Le porche garde son ombre, plus loin. Tes mains ont guidé le moulin. La marche.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Mila. Aniss pointe la &lt;emphasis&gt;marche&lt;/emphasis&gt;, du doigt. Mila attend, puis ouvre les mains. Le moulin pose ses pales sur la marche. Le courant du seuil pousse, tout net. Je le tiens. La goutte de cire rouge prend l'air, sur la marche. Le moulin attend, collé aux doigts. Le porche garde son ombre, plus loin. Tes mains ont guidé le moulin. Il tourne. [pause]</t>
+          <t>Mila. Aniss pointe la &lt;emphasis&gt;marche&lt;/emphasis&gt;, du doigt. Mila attend, puis ouvre les mains. Le moulin pose ses pales sur la marche. Le courant du seuil pousse, tout net. Je le tiens. La goutte de cire rouge prend l'air, sur la marche. Le moulin attend, collé aux doigts. Le porche garde son ombre, plus loin. Tes mains ont guidé le moulin. La marche. [pause]</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -6286,7 +6286,7 @@
 narrateur|Le moulin attend, collé aux doigts.
 maman|Le porche garde son ombre, plus loin.
 papa|Tes mains ont guidé le moulin.
-enfant-m|Il tourne.</t>
+enfant-m|La marche.</t>
         </is>
       </c>
       <c r="AX28" t="inlineStr">
@@ -6505,17 +6505,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Le nœud, Aniss. Aniss pointe le crochet du porche, du doigt. Mila attend, puis suit le doigt. Le moulin suit le nœud, tour après tour. Le jaune se tient, hors du mur. Il évite le mur. La goutte de cire rouge veille derrière le nœud. Le moulin attend, collé aux doigts. Le nœud a montré la route. Vos pieds restent au sec, aussi. Il tourne.</t>
+          <t>Le nœud, Aniss. Aniss pointe le crochet du porche, du doigt. Mila attend, puis suit le doigt. Le moulin suit le nœud, tour après tour. Le jaune se tient, hors du mur. Il évite le mur. La goutte de cire rouge veille derrière le nœud. Le moulin attend, collé aux doigts. Le nœud a montré la route. Vos pieds restent au sec, aussi. Le nœud.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;nœud&lt;/emphasis&gt;, Aniss. Aniss pointe le crochet du porche, du doigt. Mila attend, puis suit le doigt. Le moulin suit le nœud, tour après tour. Le jaune se tient, hors du mur. Il évite le mur. La goutte de cire rouge veille derrière le nœud. Le moulin attend, collé aux doigts. Le nœud a montré la route. Vos pieds restent au sec, aussi. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;nœud&lt;/emphasis&gt;, Aniss. Aniss pointe le crochet du porche, du doigt. Mila attend, puis suit le doigt. Le moulin suit le nœud, tour après tour. Le jaune se tient, hors du mur. Il évite le mur. La goutte de cire rouge veille derrière le nœud. Le moulin attend, collé aux doigts. Le nœud a montré la route. Vos pieds restent au sec, aussi. Le nœud.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;nœud&lt;/emphasis&gt;, Aniss. Aniss pointe le crochet du porche, du doigt. Mila attend, puis suit le doigt. Le moulin suit le nœud, tour après tour. Le jaune se tient, hors du mur. Il évite le mur. La goutte de cire rouge veille derrière le nœud. Le moulin attend, collé aux doigts. Le nœud a montré la route. Vos pieds restent au sec, aussi. Il tourne. [pause]</t>
+          <t>Le &lt;emphasis&gt;nœud&lt;/emphasis&gt;, Aniss. Aniss pointe le crochet du porche, du doigt. Mila attend, puis suit le doigt. Le moulin suit le nœud, tour après tour. Le jaune se tient, hors du mur. Il évite le mur. La goutte de cire rouge veille derrière le nœud. Le moulin attend, collé aux doigts. Le nœud a montré la route. Vos pieds restent au sec, aussi. Le nœud. [pause]</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -6659,7 +6659,7 @@
 narrateur|Le moulin attend, collé aux doigts.
 papa|Le nœud a montré la route.
 maman|Vos pieds restent au sec, aussi.
-enfant-m|Il tourne.</t>
+enfant-m|Le nœud.</t>
         </is>
       </c>
       <c r="AX30" t="inlineStr">
@@ -7636,17 +7636,17 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Le fil se coince entre deux barreaux froids. La grille serre trop, juste à hauteur d'Aniss. Tire-le, Aniss ! Aniss montre un écart plus bas, du doigt. Le beige racle le fer, trop près. Dis-moi où ! Aniss secoue la tête, tout petit. On ne fonce pas. Mila se tait, et son silence compte. Il montre, avec le doigt. Le crochet du loquet brille un peu. La goutte de cire rouge s'est cachée derrière un barreau. Vous faites comment, tous les deux ?</t>
+          <t>Le fil se coince entre deux barreaux froids. Le beige racle le fer, trop près des pales. Tire-le, Aniss ! Aniss enroule un tour, au lieu de tirer. Le fil se tait, puis lâche un peu. Dis nœud, alors ! Aniss montre le bas, du doigt. Plus bas. Mila se tait, les mains ouvertes. Il a enroulé, sans crier. Le crochet du loquet brille un peu. La goutte de cire rouge s'est cachée derrière un barreau. Vous faites comment, tous les deux ?</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le fil se coince entre deux barreaux froids. La grille serre trop, juste à hauteur d'Aniss. Tire-le, Aniss ! Aniss montre un écart plus bas, du doigt. Le beige racle le fer, trop près. Dis-moi où ! Aniss secoue la tête, tout petit. On ne fonce pas. Mila se tait, et son silence compte. Il montre, avec le doigt. Le crochet du loquet brille un peu. La &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; s'est cachée derrière un barreau. Vous faites comment, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le fil se coince entre deux barreaux froids. Le beige racle le fer, trop près des pales. Tire-le, Aniss ! Aniss enroule un tour, au lieu de tirer. Le fil se tait, puis lâche un peu. Dis nœud, alors ! Aniss montre le bas, du doigt. Plus bas. Mila se tait, les mains ouvertes. Il a enroulé, sans crier. Le crochet du loquet brille un peu. La &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; s'est cachée derrière un barreau. Vous faites comment, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Le fil se coince entre deux barreaux froids. La grille serre trop, juste à hauteur d'Aniss. Tire-le, Aniss ! Aniss montre un écart plus bas, du doigt. Le beige racle le fer, trop près. Dis-moi où ! Aniss secoue la tête, tout petit. On ne fonce pas. Mila se tait, et son silence compte. Il montre, avec le doigt. Le crochet du loquet brille un peu. La &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; s'est cachée derrière un barreau. Vous faites comment, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Le fil se coince entre deux barreaux froids. Le beige racle le fer, trop près des pales. Tire-le, Aniss ! Aniss enroule un tour, au lieu de tirer. Le fil se tait, puis lâche un peu. Dis nœud, alors ! Aniss montre le bas, du doigt. Plus bas. Mila se tait, les mains ouvertes. Il a enroulé, sans crier. Le crochet du loquet brille un peu. La &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; s'est cachée derrière un barreau. Vous faites comment, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
@@ -7785,15 +7785,15 @@
       <c r="AW36" t="inlineStr">
         <is>
           <t>narrateur|Le fil se coince entre deux barreaux froids.
-narrateur|La grille serre trop, juste à hauteur d'Aniss.
+narrateur|Le beige racle le fer, trop près des pales.
 copine|Tire-le, Aniss !
-narrateur|Aniss montre un écart plus bas, du doigt.
-narrateur|Le beige racle le fer, trop près.
-copine|Dis-moi où !
-narrateur|Aniss secoue la tête, tout petit.
-enfant-m|On ne fonce pas.
-narrateur|Mila se tait, et son silence compte.
-maman|Il montre, avec le doigt.
+narrateur|Aniss enroule un tour, au lieu de tirer.
+narrateur|Le fil se tait, puis lâche un peu.
+copine|Dis nœud, alors !
+narrateur|Aniss montre le bas, du doigt.
+enfant-m|Plus bas.
+narrateur|Mila se tait, les mains ouvertes.
+maman|Il a enroulé, sans crier.
 papa|Le crochet du loquet brille un peu.
 narrateur|La goutte de cire rouge s'est cachée derrière un barreau.
 papa|Vous faites comment, tous les deux ?</t>
@@ -8025,17 +8025,17 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>On attend. Aniss cherche l'écart du bas, sans presser. Mila suit le doigt, enfin, un peu. Le fil reste bas, près du bitume. Aniss glisse le bâton, sans un mot. Le fer fait toc, plus large. Toc. La goutte de cire rouge revoit le vent, ronde. Le fil attend, autour du bâton. Le bas laisse un vrai passage. Il tourne.</t>
+          <t>On attend. Aniss cherche l'écart du bas, sans presser. Mila suit le doigt, enfin, un peu. Le fil reste bas, près du bitume. Aniss glisse le bâton, sans un mot. Le fer fait toc, plus large. Toc. La goutte de cire rouge revoit le vent, ronde. Le fil attend, autour du bâton. Le bas laisse un vrai passage. En bas.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend. Aniss cherche l'écart du &lt;emphasis level="moderate"&gt;bas&lt;/emphasis&gt;, sans presser. Mila suit le doigt, enfin, un peu. Le fil reste bas, près du bitume. Aniss glisse le bâton, sans un mot. Le fer fait toc, plus large. Toc. La goutte de cire rouge revoit le vent, ronde. Le fil attend, autour du bâton. Le bas laisse un vrai passage. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend. Aniss cherche l'écart du &lt;emphasis level="moderate"&gt;bas&lt;/emphasis&gt;, sans presser. Mila suit le doigt, enfin, un peu. Le fil reste bas, près du bitume. Aniss glisse le bâton, sans un mot. Le fer fait toc, plus large. Toc. La goutte de cire rouge revoit le vent, ronde. Le fil attend, autour du bâton. Le bas laisse un vrai passage. En bas.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>On attend. Aniss cherche l'écart du &lt;emphasis&gt;bas&lt;/emphasis&gt;, sans presser. Mila suit le doigt, enfin, un peu. Le fil reste bas, près du bitume. Aniss glisse le bâton, sans un mot. Le fer fait toc, plus large. Toc. La goutte de cire rouge revoit le vent, ronde. Le fil attend, autour du bâton. Le bas laisse un vrai passage. Il tourne. [pause]</t>
+          <t>On attend. Aniss cherche l'écart du &lt;emphasis&gt;bas&lt;/emphasis&gt;, sans presser. Mila suit le doigt, enfin, un peu. Le fil reste bas, près du bitume. Aniss glisse le bâton, sans un mot. Le fer fait toc, plus large. Toc. La goutte de cire rouge revoit le vent, ronde. Le fil attend, autour du bâton. Le bas laisse un vrai passage. En bas. [pause]</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -8179,7 +8179,7 @@
 narrateur|La goutte de cire rouge revoit le vent, ronde.
 narrateur|Le fil attend, autour du bâton.
 papa|Le bas laisse un vrai passage.
-enfant-m|Il tourne.</t>
+enfant-m|En bas.</t>
         </is>
       </c>
       <c r="AX38" t="inlineStr">
@@ -8211,17 +8211,17 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Le moulin pose une pale sur le fer. Tourne. Il est arrivé. Les barreaux ont failli garder le papier. Le bas a laissé le passage. Le fil pend, un peu humide, contre le fer. Un rai rouge s'allonge sur le bitume, puis s'arrête. Le fil laisse la goutte de cire rouge au fer.</t>
+          <t>Le moulin pose une pale sur le fer. Tourne. Il est arrivé. Le fil a failli rester dans le fer. Le bas a laissé le passage. Le fil pend, un peu humide, contre le fer. Un fil beige tremble, puis se tait. Le fil laisse la goutte de cire rouge au fer.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le moulin pose une pale sur le fer. Tourne. Il est arrivé. Les barreaux ont failli garder le papier. Le bas a laissé le passage. Le fil pend, un peu humide, contre le fer. Un rai rouge s'allonge sur le bitume, puis s'arrête. Le fil laisse la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; au fer.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le moulin pose une pale sur le fer. Tourne. Il est arrivé. Le fil a failli rester dans le fer. Le bas a laissé le passage. Le fil pend, un peu humide, contre le fer. Un fil beige tremble, puis se tait. Le fil laisse la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; au fer.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le moulin pose une pale sur le fer. Tourne. Il est arrivé. Les barreaux ont failli garder le papier. Le bas a laissé le passage. Le fil pend, un peu humide, contre le fer. Un rai rouge s'allonge sur le bitume, puis s'arrête. Le fil laisse la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; au fer.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le moulin pose une pale sur le fer. Tourne. Il est arrivé. Le fil a failli rester dans le fer. Le bas a laissé le passage. Le fil pend, un peu humide, contre le fer. Un fil beige tremble, puis se tait. Le fil laisse la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; au fer.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -8362,10 +8362,10 @@
           <t>narrateur|Le moulin pose une pale sur le fer.
 enfant-m|Tourne.
 copine|Il est arrivé.
-narrateur|Les barreaux ont failli garder le papier.
+narrateur|Le fil a failli rester dans le fer.
 papa|Le bas a laissé le passage.
 narrateur|Le fil pend, un peu humide, contre le fer.
-narrateur|Un rai rouge s'allonge sur le bitume, puis s'arrête.
+narrateur|Un fil beige tremble, puis se tait.
 narrateur|Le fil laisse la goutte de cire rouge au fer.</t>
         </is>
       </c>
@@ -8398,17 +8398,17 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Pour toi. Mila ouvre les deux mains, tout près. Aniss pose le jaune contre ses paumes. Le fil guide le papier vers Mila. Mila vise l'écart, Aniss pousse le bâton. Il passe ! La goutte de cire rouge échappe au fer, ronde. Le fil attend, autour du bâton. Tes mains ont trouvé le fer. Il l'a tendu, d'abord. Il tourne.</t>
+          <t>Pour toi. Mila ouvre les deux mains, tout près. Aniss pose le jaune contre ses paumes. Le fil guide le papier vers Mila. Mila vise l'écart, Aniss pousse le bâton. Il passe ! La goutte de cire rouge échappe au fer, ronde. Le fil attend, autour du bâton. Tes mains ont trouvé le fer. Il l'a tendu, d'abord. Tes mains.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Pour toi. Mila ouvre les deux &lt;emphasis level="moderate"&gt;mains&lt;/emphasis&gt;, tout près. Aniss pose le jaune contre ses paumes. Le fil guide le papier vers Mila. Mila vise l'écart, Aniss pousse le bâton. Il passe ! La goutte de cire rouge échappe au fer, ronde. Le fil attend, autour du bâton. Tes mains ont trouvé le fer. Il l'a tendu, d'abord. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Pour toi. Mila ouvre les deux &lt;emphasis level="moderate"&gt;mains&lt;/emphasis&gt;, tout près. Aniss pose le jaune contre ses paumes. Le fil guide le papier vers Mila. Mila vise l'écart, Aniss pousse le bâton. Il passe ! La goutte de cire rouge échappe au fer, ronde. Le fil attend, autour du bâton. Tes mains ont trouvé le fer. Il l'a tendu, d'abord. Tes mains.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Pour toi. Mila ouvre les deux &lt;emphasis&gt;mains&lt;/emphasis&gt;, tout près. Aniss pose le jaune contre ses paumes. Le fil guide le papier vers Mila. Mila vise l'écart, Aniss pousse le bâton. Il passe ! La goutte de cire rouge échappe au fer, ronde. Le fil attend, autour du bâton. Tes mains ont trouvé le fer. Il l'a tendu, d'abord. Il tourne. [pause]</t>
+          <t>Pour toi. Mila ouvre les deux &lt;emphasis&gt;mains&lt;/emphasis&gt;, tout près. Aniss pose le jaune contre ses paumes. Le fil guide le papier vers Mila. Mila vise l'écart, Aniss pousse le bâton. Il passe ! La goutte de cire rouge échappe au fer, ronde. Le fil attend, autour du bâton. Tes mains ont trouvé le fer. Il l'a tendu, d'abord. Tes mains. [pause]</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -8552,7 +8552,7 @@
 narrateur|Le fil attend, autour du bâton.
 maman|Tes mains ont trouvé le fer.
 papa|Il l'a tendu, d'abord.
-enfant-m|Il tourne.</t>
+enfant-m|Tes mains.</t>
         </is>
       </c>
       <c r="AX40" t="inlineStr">
@@ -8584,17 +8584,17 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Le jaune s'est glissé jusqu'au barreau. Aniss l'a tendu, tout seul. Tu as tendu, d'abord. Les barreaux ont failli garder le papier. Venez, le moulin est près de la grille. Le fil pend, un peu humide, contre le fer. Au muret, ça sent la cire, tiède. Les mains de Mila chauffent la goutte de cire rouge.</t>
+          <t>Le jaune s'est glissé jusqu'au barreau. Aniss l'a tendu, tout seul. Tu as tendu, d'abord. Le fil a failli rester dans le fer. Venez, le moulin est près de la grille. Le fil pend, un peu humide, contre le fer. Une pale sèche, contre le fer. Les mains de Mila chauffent la goutte de cire rouge.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jaune s'est glissé jusqu'au barreau. Aniss l'a tendu, tout seul. Tu as tendu, d'abord. Les barreaux ont failli garder le papier. Venez, le moulin est près de la grille. Le fil pend, un peu humide, contre le fer. Au muret, ça sent la cire, tiède. Les mains de Mila chauffent la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jaune s'est glissé jusqu'au barreau. Aniss l'a tendu, tout seul. Tu as tendu, d'abord. Le fil a failli rester dans le fer. Venez, le moulin est près de la grille. Le fil pend, un peu humide, contre le fer. Une pale sèche, contre le fer. Les mains de Mila chauffent la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jaune s'est glissé jusqu'au barreau. Aniss l'a tendu, tout seul. Tu as tendu, d'abord. Les barreaux ont failli garder le papier. Venez, le moulin est près de la grille. Le fil pend, un peu humide, contre le fer. Au muret, ça sent la cire, tiède. Les mains de Mila chauffent la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jaune s'est glissé jusqu'au barreau. Aniss l'a tendu, tout seul. Tu as tendu, d'abord. Le fil a failli rester dans le fer. Venez, le moulin est près de la grille. Le fil pend, un peu humide, contre le fer. Une pale sèche, contre le fer. Les mains de Mila chauffent la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -8735,10 +8735,10 @@
           <t>narrateur|Le jaune s'est glissé jusqu'au barreau.
 copine|Aniss l'a tendu, tout seul.
 papa|Tu as tendu, d'abord.
-narrateur|Les barreaux ont failli garder le papier.
+narrateur|Le fil a failli rester dans le fer.
 maman|Venez, le moulin est près de la grille.
 narrateur|Le fil pend, un peu humide, contre le fer.
-narrateur|Au muret, ça sent la cire, tiède.
+narrateur|Une pale sèche, contre le fer.
 narrateur|Les mains de Mila chauffent la goutte de cire rouge.</t>
         </is>
       </c>
@@ -8771,17 +8771,17 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Le crochet, Aniss. Aniss lève le jaune, sans un mot. Mila attend, puis suit sa main. Le fil s'enroule au crochet du loquet. Une pale racle le fer, puis se libère. Il tient. La goutte de cire rouge reprend le rai, petite. Le fil attend, autour du bâton. Le loquet a gardé le papier. Les barreaux peuvent dormir, plus loin. Il tourne.</t>
+          <t>Le crochet, Aniss. Aniss lève le jaune, sans un mot. Mila attend, puis suit sa main. Le fil s'enroule au crochet du loquet. Une pale racle le fer, puis se libère. Il tient. La goutte de cire rouge reprend le rai, petite. Le fil attend, autour du bâton. Le loquet a gardé le papier. Les barreaux peuvent dormir, plus loin. Au crochet.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;crochet&lt;/emphasis&gt;, Aniss. Aniss lève le jaune, sans un mot. Mila attend, puis suit sa main. Le fil s'enroule au crochet du loquet. Une pale racle le fer, puis se libère. Il tient. La goutte de cire rouge reprend le rai, petite. Le fil attend, autour du bâton. Le loquet a gardé le papier. Les barreaux peuvent dormir, plus loin. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;crochet&lt;/emphasis&gt;, Aniss. Aniss lève le jaune, sans un mot. Mila attend, puis suit sa main. Le fil s'enroule au crochet du loquet. Une pale racle le fer, puis se libère. Il tient. La goutte de cire rouge reprend le rai, petite. Le fil attend, autour du bâton. Le loquet a gardé le papier. Les barreaux peuvent dormir, plus loin. Au crochet.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;crochet&lt;/emphasis&gt;, Aniss. Aniss lève le jaune, sans un mot. Mila attend, puis suit sa main. Le fil s'enroule au crochet du loquet. Une pale racle le fer, puis se libère. Il tient. La goutte de cire rouge reprend le rai, petite. Le fil attend, autour du bâton. Le loquet a gardé le papier. Les barreaux peuvent dormir, plus loin. Il tourne. [pause]</t>
+          <t>Le &lt;emphasis&gt;crochet&lt;/emphasis&gt;, Aniss. Aniss lève le jaune, sans un mot. Mila attend, puis suit sa main. Le fil s'enroule au crochet du loquet. Une pale racle le fer, puis se libère. Il tient. La goutte de cire rouge reprend le rai, petite. Le fil attend, autour du bâton. Le loquet a gardé le papier. Les barreaux peuvent dormir, plus loin. Au crochet. [pause]</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -8925,7 +8925,7 @@
 narrateur|Le fil attend, autour du bâton.
 papa|Le loquet a gardé le papier.
 maman|Les barreaux peuvent dormir, plus loin.
-enfant-m|Il tourne.</t>
+enfant-m|Au crochet.</t>
         </is>
       </c>
       <c r="AX42" t="inlineStr">
@@ -8957,17 +8957,17 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Le jaune pend au crochet, tout droit. On a posé le moulin. Le crochet a tenu, tout droit. Les barreaux ont failli garder le papier. Essuyez vos mains, tout près. Le fil pend, un peu humide, contre le fer. Au loin, le bus se tait. Le loquet garde la goutte de cire rouge, minuscule.</t>
+          <t>Le jaune pend au crochet, tout droit. On a posé le moulin. Le crochet a tenu, tout droit. Le fil a failli rester dans le fer. Essuyez vos mains, tout près. Le fil pend, un peu humide, contre le fer. Sur le bitume, une trace d'eau, mince. Le loquet garde la goutte de cire rouge, minuscule.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jaune pend au crochet, tout droit. On a posé le moulin. Le crochet a tenu, tout droit. Les barreaux ont failli garder le papier. Essuyez vos mains, tout près. Le fil pend, un peu humide, contre le fer. Au loin, le bus se tait. Le loquet garde la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;, minuscule.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jaune pend au crochet, tout droit. On a posé le moulin. Le crochet a tenu, tout droit. Le fil a failli rester dans le fer. Essuyez vos mains, tout près. Le fil pend, un peu humide, contre le fer. Sur le bitume, une trace d'eau, mince. Le loquet garde la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;, minuscule.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jaune pend au crochet, tout droit. On a posé le moulin. Le crochet a tenu, tout droit. Les barreaux ont failli garder le papier. Essuyez vos mains, tout près. Le fil pend, un peu humide, contre le fer. Au loin, le bus se tait. Le loquet garde la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;, minuscule.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jaune pend au crochet, tout droit. On a posé le moulin. Le crochet a tenu, tout droit. Le fil a failli rester dans le fer. Essuyez vos mains, tout près. Le fil pend, un peu humide, contre le fer. Sur le bitume, une trace d'eau, mince. Le loquet garde la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;, minuscule.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -9108,10 +9108,10 @@
           <t>narrateur|Le jaune pend au crochet, tout droit.
 copine|On a posé le moulin.
 papa|Le crochet a tenu, tout droit.
-narrateur|Les barreaux ont failli garder le papier.
+narrateur|Le fil a failli rester dans le fer.
 maman|Essuyez vos mains, tout près.
 narrateur|Le fil pend, un peu humide, contre le fer.
-narrateur|Au loin, le bus se tait.
+narrateur|Sur le bitume, une trace d'eau, mince.
 narrateur|Le loquet garde la goutte de cire rouge, minuscule.</t>
         </is>
       </c>
@@ -9144,17 +9144,17 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Le fil traîne dans l'eau, trop vite. L'eau est trop grande. Une feuille jaune part, plus bas. Tire, Aniss ! Aniss ramène le beige, sans presser. L'eau frappe la dalle, puis rebondit. On ne fonce pas. Mila referme la bouche. Son silence compte, comme une réponse. La dalle tient le courant. On reste près du caniveau, tous les deux. La goutte de cire rouge s'est ternie, trop près de l'eau. Vous faites comment, tous les deux ?</t>
+          <t>Le fil traîne dans l'eau, trop vite. L'eau est trop grande. Le beige s'alourdit, puis tire le papier. Tire, Aniss ! Aniss enroule le fil, tour après tour. L'eau frappe la dalle, puis rebondit. Attends l'eau. Mila referme la bouche. Elle pose une main sur le fil, sans tirer. La dalle tient le courant. On reste près du caniveau, tous les deux. La goutte de cire rouge s'est ternie, trop près de l'eau. Vous faites comment, tous les deux ?</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le fil traîne dans l'eau, trop vite. L'eau est trop grande. Une feuille jaune part, plus bas. Tire, Aniss ! Aniss ramène le beige, sans presser. L'eau frappe la dalle, puis rebondit. On ne fonce pas. Mila referme la bouche. Son silence compte, comme une réponse. La dalle tient le courant. On reste près du caniveau, tous les deux. La &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; s'est ternie, trop près de l'eau. Vous faites comment, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le fil traîne dans l'eau, trop vite. L'eau est trop grande. Le beige s'alourdit, puis tire le papier. Tire, Aniss ! Aniss enroule le fil, tour après tour. L'eau frappe la dalle, puis rebondit. Attends l'eau. Mila referme la bouche. Elle pose une main sur le fil, sans tirer. La dalle tient le courant. On reste près du caniveau, tous les deux. La &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; s'est ternie, trop près de l'eau. Vous faites comment, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Le fil traîne dans l'eau, trop vite. L'eau est trop grande. Une feuille jaune part, plus bas. Tire, Aniss ! Aniss ramène le beige, sans presser. L'eau frappe la dalle, puis rebondit. On ne fonce pas. Mila referme la bouche. Son silence compte, comme une réponse. La dalle tient le courant. On reste près du caniveau, tous les deux. La &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; s'est ternie, trop près de l'eau. Vous faites comment, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Le fil traîne dans l'eau, trop vite. L'eau est trop grande. Le beige s'alourdit, puis tire le papier. Tire, Aniss ! Aniss enroule le fil, tour après tour. L'eau frappe la dalle, puis rebondit. Attends l'eau. Mila referme la bouche. Elle pose une main sur le fil, sans tirer. La dalle tient le courant. On reste près du caniveau, tous les deux. La &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; s'est ternie, trop près de l'eau. Vous faites comment, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -9294,13 +9294,13 @@
         <is>
           <t>narrateur|Le fil traîne dans l'eau, trop vite.
 copine|L'eau est trop grande.
-narrateur|Une feuille jaune part, plus bas.
+narrateur|Le beige s'alourdit, puis tire le papier.
 copine|Tire, Aniss !
-narrateur|Aniss ramène le beige, sans presser.
+narrateur|Aniss enroule le fil, tour après tour.
 narrateur|L'eau frappe la dalle, puis rebondit.
-enfant-m|On ne fonce pas.
+enfant-m|Attends l'eau.
 narrateur|Mila referme la bouche.
-narrateur|Son silence compte, comme une réponse.
+narrateur|Elle pose une main sur le fil, sans tirer.
 maman|La dalle tient le courant.
 papa|On reste près du caniveau, tous les deux.
 narrateur|La goutte de cire rouge s'est ternie, trop près de l'eau.
@@ -9533,17 +9533,17 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>On attend l'eau. Aniss s'assoit près du caniveau, sans presser. Mila s'assoit aussi, les genoux contre lui. Le fil sèche contre la dalle. L'eau frappe, puis la feuille s'arrête. Maintenant. La goutte de cire rouge sèche, ronde, sur la dalle. Le fil attend, autour du bâton. La dalle a cassé le courant. Vous avez laissé l'eau finir. Il tourne.</t>
+          <t>On attend l'eau. Aniss s'assoit près du caniveau, sans presser. Mila s'assoit aussi, les genoux contre lui. Le fil sèche contre la dalle. L'eau frappe, puis la feuille s'arrête. Maintenant. La goutte de cire rouge sèche, ronde, sur la dalle. Le fil attend, autour du bâton. La dalle a cassé le courant. Vous avez laissé l'eau finir. La dalle.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend l'eau. Aniss s'assoit près du caniveau, sans presser. Mila s'assoit aussi, les genoux contre lui. Le fil sèche contre la &lt;emphasis level="moderate"&gt;dalle&lt;/emphasis&gt;. L'eau frappe, puis la feuille s'arrête. Maintenant. La goutte de cire rouge sèche, ronde, sur la dalle. Le fil attend, autour du bâton. La dalle a cassé le courant. Vous avez laissé l'eau finir. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend l'eau. Aniss s'assoit près du caniveau, sans presser. Mila s'assoit aussi, les genoux contre lui. Le fil sèche contre la &lt;emphasis level="moderate"&gt;dalle&lt;/emphasis&gt;. L'eau frappe, puis la feuille s'arrête. Maintenant. La goutte de cire rouge sèche, ronde, sur la dalle. Le fil attend, autour du bâton. La dalle a cassé le courant. Vous avez laissé l'eau finir. La dalle.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>On attend l'eau. Aniss s'assoit près du caniveau, sans presser. Mila s'assoit aussi, les genoux contre lui. Le fil sèche contre la &lt;emphasis&gt;dalle&lt;/emphasis&gt;. L'eau frappe, puis la feuille s'arrête. Maintenant. La goutte de cire rouge sèche, ronde, sur la dalle. Le fil attend, autour du bâton. La dalle a cassé le courant. Vous avez laissé l'eau finir. Il tourne. [pause]</t>
+          <t>On attend l'eau. Aniss s'assoit près du caniveau, sans presser. Mila s'assoit aussi, les genoux contre lui. Le fil sèche contre la &lt;emphasis&gt;dalle&lt;/emphasis&gt;. L'eau frappe, puis la feuille s'arrête. Maintenant. La goutte de cire rouge sèche, ronde, sur la dalle. Le fil attend, autour du bâton. La dalle a cassé le courant. Vous avez laissé l'eau finir. La dalle. [pause]</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -9687,7 +9687,7 @@
 narrateur|Le fil attend, autour du bâton.
 papa|La dalle a cassé le courant.
 maman|Vous avez laissé l'eau finir.
-enfant-m|Il tourne.</t>
+enfant-m|La dalle.</t>
         </is>
       </c>
       <c r="AX46" t="inlineStr">
@@ -9719,17 +9719,17 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Le jaune rejoint la grille, un peu mouillé. On a attendu l'eau. Le caniveau n'a plus pris vos bras. L'eau a failli emporter la pale. Rentrez le fil, après la grille. Le fil pend, un peu humide, contre le fer. Un rai rouge s'allonge sur le bitume, puis s'arrête. L'eau n'a pas pris la goutte de cire rouge.</t>
+          <t>Le jaune rejoint la grille, un peu mouillé. On a attendu l'eau. Le caniveau n'a plus pris vos bras. Le fil a failli partir avec l'eau. Rentrez le fil, après la grille. Le fil pend, un peu humide, contre le fer. Un fil beige tremble, puis se tait. L'eau n'a pas pris la goutte de cire rouge.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jaune rejoint la grille, un peu mouillé. On a attendu l'eau. Le caniveau n'a plus pris vos bras. L'eau a failli emporter la pale. Rentrez le fil, après la grille. Le fil pend, un peu humide, contre le fer. Un rai rouge s'allonge sur le bitume, puis s'arrête. L'eau n'a pas pris la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jaune rejoint la grille, un peu mouillé. On a attendu l'eau. Le caniveau n'a plus pris vos bras. Le fil a failli partir avec l'eau. Rentrez le fil, après la grille. Le fil pend, un peu humide, contre le fer. Un fil beige tremble, puis se tait. L'eau n'a pas pris la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jaune rejoint la grille, un peu mouillé. On a attendu l'eau. Le caniveau n'a plus pris vos bras. L'eau a failli emporter la pale. Rentrez le fil, après la grille. Le fil pend, un peu humide, contre le fer. Un rai rouge s'allonge sur le bitume, puis s'arrête. L'eau n'a pas pris la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jaune rejoint la grille, un peu mouillé. On a attendu l'eau. Le caniveau n'a plus pris vos bras. Le fil a failli partir avec l'eau. Rentrez le fil, après la grille. Le fil pend, un peu humide, contre le fer. Un fil beige tremble, puis se tait. L'eau n'a pas pris la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -9870,10 +9870,10 @@
           <t>narrateur|Le jaune rejoint la grille, un peu mouillé.
 copine|On a attendu l'eau.
 papa|Le caniveau n'a plus pris vos bras.
-narrateur|L'eau a failli emporter la pale.
+narrateur|Le fil a failli partir avec l'eau.
 maman|Rentrez le fil, après la grille.
 narrateur|Le fil pend, un peu humide, contre le fer.
-narrateur|Un rai rouge s'allonge sur le bitume, puis s'arrête.
+narrateur|Un fil beige tremble, puis se tait.
 narrateur|L'eau n'a pas pris la goutte de cire rouge.</t>
         </is>
       </c>
@@ -9906,17 +9906,17 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Tes mains, Aniss. Aniss tend le fil, tout près. Mila tire avec lui, sans presser. Le fil part au bout des mains de Mila. Le papier passe au-dessus de l'eau. On tient ensemble. La goutte de cire rouge tremble au bout du fil. Le fil attend, autour du bâton. Vos mains suffisent, toutes les deux. L'eau restera après. Il tourne.</t>
+          <t>Tes mains, Aniss. Aniss tend le fil, tout près. Mila tire avec lui, sans presser. Le fil part au bout des mains de Mila. Le papier passe au-dessus de l'eau. On tient ensemble. La goutte de cire rouge tremble au bout du fil. Le fil attend, autour du bâton. Vos mains suffisent, toutes les deux. L'eau restera après. On tient.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tes mains, Aniss. Aniss tend le &lt;emphasis level="moderate"&gt;fil&lt;/emphasis&gt;, tout près. Mila tire avec lui, sans presser. Le fil part au bout des mains de Mila. Le papier passe au-dessus de l'eau. On tient ensemble. La goutte de cire rouge tremble au bout du fil. Le fil attend, autour du bâton. Vos mains suffisent, toutes les deux. L'eau restera après. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tes mains, Aniss. Aniss tend le &lt;emphasis level="moderate"&gt;fil&lt;/emphasis&gt;, tout près. Mila tire avec lui, sans presser. Le fil part au bout des mains de Mila. Le papier passe au-dessus de l'eau. On tient ensemble. La goutte de cire rouge tremble au bout du fil. Le fil attend, autour du bâton. Vos mains suffisent, toutes les deux. L'eau restera après. On tient.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Tes mains, Aniss. Aniss tend le &lt;emphasis&gt;fil&lt;/emphasis&gt;, tout près. Mila tire avec lui, sans presser. Le fil part au bout des mains de Mila. Le papier passe au-dessus de l'eau. On tient ensemble. La goutte de cire rouge tremble au bout du fil. Le fil attend, autour du bâton. Vos mains suffisent, toutes les deux. L'eau restera après. Il tourne. [pause]</t>
+          <t>Tes mains, Aniss. Aniss tend le &lt;emphasis&gt;fil&lt;/emphasis&gt;, tout près. Mila tire avec lui, sans presser. Le fil part au bout des mains de Mila. Le papier passe au-dessus de l'eau. On tient ensemble. La goutte de cire rouge tremble au bout du fil. Le fil attend, autour du bâton. Vos mains suffisent, toutes les deux. L'eau restera après. On tient. [pause]</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -10060,7 +10060,7 @@
 narrateur|Le fil attend, autour du bâton.
 maman|Vos mains suffisent, toutes les deux.
 papa|L'eau restera après.
-enfant-m|Il tourne.</t>
+enfant-m|On tient.</t>
         </is>
       </c>
       <c r="AX48" t="inlineStr">
@@ -10092,17 +10092,17 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Le fil pose le moulin contre le fer. On tenait, tous les deux. Je remporte le fil, tout à l'heure. L'eau a failli emporter la pale. La grille vous attend. Le fil pend, un peu humide, contre le fer. Au muret, ça sent la cire, tiède. Le fil tendu montre la goutte de cire rouge au soleil.</t>
+          <t>Le fil pose le moulin contre le fer. On tenait, tous les deux. Je remporte le fil, tout à l'heure. Le fil a failli partir avec l'eau. La grille vous attend. Le fil pend, un peu humide, contre le fer. Une pale sèche, contre le fer. Le fil tendu montre la goutte de cire rouge au soleil.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le fil pose le moulin contre le fer. On tenait, tous les deux. Je remporte le fil, tout à l'heure. L'eau a failli emporter la pale. La grille vous attend. Le fil pend, un peu humide, contre le fer. Au muret, ça sent la cire, tiède. Le fil tendu montre la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; au soleil.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le fil pose le moulin contre le fer. On tenait, tous les deux. Je remporte le fil, tout à l'heure. Le fil a failli partir avec l'eau. La grille vous attend. Le fil pend, un peu humide, contre le fer. Une pale sèche, contre le fer. Le fil tendu montre la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; au soleil.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le fil pose le moulin contre le fer. On tenait, tous les deux. Je remporte le fil, tout à l'heure. L'eau a failli emporter la pale. La grille vous attend. Le fil pend, un peu humide, contre le fer. Au muret, ça sent la cire, tiède. Le fil tendu montre la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; au soleil.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le fil pose le moulin contre le fer. On tenait, tous les deux. Je remporte le fil, tout à l'heure. Le fil a failli partir avec l'eau. La grille vous attend. Le fil pend, un peu humide, contre le fer. Une pale sèche, contre le fer. Le fil tendu montre la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; au soleil.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -10243,10 +10243,10 @@
           <t>narrateur|Le fil pose le moulin contre le fer.
 copine|On tenait, tous les deux.
 papa|Je remporte le fil, tout à l'heure.
-narrateur|L'eau a failli emporter la pale.
+narrateur|Le fil a failli partir avec l'eau.
 maman|La grille vous attend.
 narrateur|Le fil pend, un peu humide, contre le fer.
-narrateur|Au muret, ça sent la cire, tiède.
+narrateur|Une pale sèche, contre le fer.
 narrateur|Le fil tendu montre la goutte de cire rouge au soleil.</t>
         </is>
       </c>
@@ -10279,17 +10279,17 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Le bord, d'abord. Mila tend la pierre sèche vers Aniss. Aniss marche, sans un mot. Le fil suit le bord sec. Une goutte rejoint le fond, puis se tait. C'est doux. La goutte de cire rouge reste au sec, sur le bord. Le fil attend, autour du bâton. L'eau garde son souffle, plus loin. Le bord a laissé le papier. Il tourne.</t>
+          <t>Le bord, d'abord. Mila tend la pierre sèche vers Aniss. Aniss marche, sans un mot. Le fil suit le bord sec. Une goutte rejoint le fond, puis se tait. C'est doux. La goutte de cire rouge reste au sec, sur le bord. Le fil attend, autour du bâton. L'eau garde son souffle, plus loin. Le bord a laissé le papier. Au sec.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;bord&lt;/emphasis&gt;, d'abord. Mila tend la pierre sèche vers Aniss. Aniss marche, sans un mot. Le fil suit le bord sec. Une goutte rejoint le fond, puis se tait. C'est doux. La goutte de cire rouge reste au sec, sur le bord. Le fil attend, autour du bâton. L'eau garde son souffle, plus loin. Le bord a laissé le papier. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;bord&lt;/emphasis&gt;, d'abord. Mila tend la pierre sèche vers Aniss. Aniss marche, sans un mot. Le fil suit le bord sec. Une goutte rejoint le fond, puis se tait. C'est doux. La goutte de cire rouge reste au sec, sur le bord. Le fil attend, autour du bâton. L'eau garde son souffle, plus loin. Le bord a laissé le papier. Au sec.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;bord&lt;/emphasis&gt;, d'abord. Mila tend la pierre sèche vers Aniss. Aniss marche, sans un mot. Le fil suit le bord sec. Une goutte rejoint le fond, puis se tait. C'est doux. La goutte de cire rouge reste au sec, sur le bord. Le fil attend, autour du bâton. L'eau garde son souffle, plus loin. Le bord a laissé le papier. Il tourne. [pause]</t>
+          <t>Le &lt;emphasis&gt;bord&lt;/emphasis&gt;, d'abord. Mila tend la pierre sèche vers Aniss. Aniss marche, sans un mot. Le fil suit le bord sec. Une goutte rejoint le fond, puis se tait. C'est doux. La goutte de cire rouge reste au sec, sur le bord. Le fil attend, autour du bâton. L'eau garde son souffle, plus loin. Le bord a laissé le papier. Au sec. [pause]</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -10433,7 +10433,7 @@
 narrateur|Le fil attend, autour du bâton.
 maman|L'eau garde son souffle, plus loin.
 papa|Le bord a laissé le papier.
-enfant-m|Il tourne.</t>
+enfant-m|Au sec.</t>
         </is>
       </c>
       <c r="AX50" t="inlineStr">
@@ -10465,17 +10465,17 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Les mains d'Aniss laissent le jaune contre le fer. C'était plus facile, là. Tes bras ont guidé le moulin. L'eau a failli emporter la pale. Le barreau gardera son ombre. Le fil pend, un peu humide, contre le fer. Au loin, le bus se tait. Le bord a sauvé la goutte de cire rouge, tiède.</t>
+          <t>Les mains d'Aniss laissent le jaune contre le fer. C'était plus facile, là. Tes bras ont guidé le moulin. Le fil a failli partir avec l'eau. Le barreau gardera son ombre. Le fil pend, un peu humide, contre le fer. Sur le bitume, une trace d'eau, mince. Le bord a sauvé la goutte de cire rouge, tiède.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les mains d'Aniss laissent le jaune contre le fer. C'était plus facile, là. Tes bras ont guidé le moulin. L'eau a failli emporter la pale. Le barreau gardera son ombre. Le fil pend, un peu humide, contre le fer. Au loin, le bus se tait. Le bord a sauvé la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;, tiède.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les mains d'Aniss laissent le jaune contre le fer. C'était plus facile, là. Tes bras ont guidé le moulin. Le fil a failli partir avec l'eau. Le barreau gardera son ombre. Le fil pend, un peu humide, contre le fer. Sur le bitume, une trace d'eau, mince. Le bord a sauvé la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;, tiède.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les mains d'Aniss laissent le jaune contre le fer. C'était plus facile, là. Tes bras ont guidé le moulin. L'eau a failli emporter la pale. Le barreau gardera son ombre. Le fil pend, un peu humide, contre le fer. Au loin, le bus se tait. Le bord a sauvé la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;, tiède.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les mains d'Aniss laissent le jaune contre le fer. C'était plus facile, là. Tes bras ont guidé le moulin. Le fil a failli partir avec l'eau. Le barreau gardera son ombre. Le fil pend, un peu humide, contre le fer. Sur le bitume, une trace d'eau, mince. Le bord a sauvé la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;, tiède.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -10616,10 +10616,10 @@
           <t>narrateur|Les mains d'Aniss laissent le jaune contre le fer.
 copine|C'était plus facile, là.
 papa|Tes bras ont guidé le moulin.
-narrateur|L'eau a failli emporter la pale.
+narrateur|Le fil a failli partir avec l'eau.
 maman|Le barreau gardera son ombre.
 narrateur|Le fil pend, un peu humide, contre le fer.
-narrateur|Au loin, le bus se tait.
+narrateur|Sur le bitume, une trace d'eau, mince.
 narrateur|Le bord a sauvé la goutte de cire rouge, tiède.</t>
         </is>
       </c>
@@ -10652,17 +10652,17 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Le fil pend, trop lourd, sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis vent ! Aniss pointe la porte, du doigt. Le porche garde l'air, trop fermé. On ne fonce pas. Mila se tait, les joues gonflées. Son silence compte, comme une réponse. Tes yeux vont plus loin, Aniss. La marche du seuil est sèche. La goutte de cire rouge s'est éteinte, dans l'ombre. Vous faites comment, tous les deux ?</t>
+          <t>Le fil pend, trop lourd, sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis nœud ! Aniss enroule le fil autour du doigt. Le beige reste mou, sans air. La porte. Mila se tait, les joues dégonflées. Elle suit le doigt, vers le seuil. Tes yeux vont plus loin, Aniss. La marche du seuil est sèche. La goutte de cire rouge s'est éteinte, dans l'ombre. Vous faites comment, tous les deux ?</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le fil pend, trop lourd, sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis vent ! Aniss pointe la porte, du doigt. Le porche garde l'air, trop fermé. On ne fonce pas. Mila se tait, les joues gonflées. Son silence compte, comme une réponse. Tes yeux vont plus loin, Aniss. La marche du seuil est sèche. La &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; s'est éteinte, dans l'ombre. Vous faites comment, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le fil pend, trop lourd, sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis nœud ! Aniss enroule le fil autour du doigt. Le beige reste mou, sans air. La porte. Mila se tait, les joues dégonflées. Elle suit le doigt, vers le seuil. Tes yeux vont plus loin, Aniss. La marche du seuil est sèche. La &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; s'est éteinte, dans l'ombre. Vous faites comment, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Le fil pend, trop lourd, sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis vent ! Aniss pointe la porte, du doigt. Le porche garde l'air, trop fermé. On ne fonce pas. Mila se tait, les joues gonflées. Son silence compte, comme une réponse. Tes yeux vont plus loin, Aniss. La marche du seuil est sèche. La &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; s'est éteinte, dans l'ombre. Vous faites comment, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Le fil pend, trop lourd, sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis nœud ! Aniss enroule le fil autour du doigt. Le beige reste mou, sans air. La porte. Mila se tait, les joues dégonflées. Elle suit le doigt, vers le seuil. Tes yeux vont plus loin, Aniss. La marche du seuil est sèche. La &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; s'est éteinte, dans l'ombre. Vous faites comment, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -10803,12 +10803,12 @@
           <t>narrateur|Le fil pend, trop lourd, sous le porche.
 copine|Ça ne tourne plus, Aniss !
 narrateur|Mila souffle trop vite, trop fort.
-copine|Dis vent !
-narrateur|Aniss pointe la porte, du doigt.
-narrateur|Le porche garde l'air, trop fermé.
-enfant-m|On ne fonce pas.
-narrateur|Mila se tait, les joues gonflées.
-narrateur|Son silence compte, comme une réponse.
+copine|Dis nœud !
+narrateur|Aniss enroule le fil autour du doigt.
+narrateur|Le beige reste mou, sans air.
+enfant-m|La porte.
+narrateur|Mila se tait, les joues dégonflées.
+narrateur|Elle suit le doigt, vers le seuil.
 maman|Tes yeux vont plus loin, Aniss.
 papa|La marche du seuil est sèche.
 narrateur|La goutte de cire rouge s'est éteinte, dans l'ombre.
@@ -11041,17 +11041,17 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Le vent, d'abord. J'ouvre un peu, à votre hauteur. Aniss attend, Mila tient le jaune. Le fil prend le vent de la porte. Une pale part, sans un mot. Ça tient ! La goutte de cire rouge file dans le courant, ronde. Le fil attend, autour du bâton. La porte a donné le courant. Aniss a poussé, sans crier. Il tourne.</t>
+          <t>Le vent, d'abord. J'ouvre un peu, à votre hauteur. Aniss attend, Mila tient le jaune. Le fil prend le vent de la porte. Une pale part, sans un mot. Ça tient ! La goutte de cire rouge file dans le courant, ronde. Le fil attend, autour du bâton. La porte a donné le courant. Aniss a poussé, sans crier. Le vent.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;vent&lt;/emphasis&gt;, d'abord. J'ouvre un peu, à votre hauteur. Aniss attend, Mila tient le jaune. Le fil prend le vent de la porte. Une pale part, sans un mot. Ça tient ! La goutte de cire rouge file dans le courant, ronde. Le fil attend, autour du bâton. La porte a donné le courant. Aniss a poussé, sans crier. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;vent&lt;/emphasis&gt;, d'abord. J'ouvre un peu, à votre hauteur. Aniss attend, Mila tient le jaune. Le fil prend le vent de la porte. Une pale part, sans un mot. Ça tient ! La goutte de cire rouge file dans le courant, ronde. Le fil attend, autour du bâton. La porte a donné le courant. Aniss a poussé, sans crier. Le vent.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;vent&lt;/emphasis&gt;, d'abord. J'ouvre un peu, à votre hauteur. Aniss attend, Mila tient le jaune. Le fil prend le vent de la porte. Une pale part, sans un mot. Ça tient ! La goutte de cire rouge file dans le courant, ronde. Le fil attend, autour du bâton. La porte a donné le courant. Aniss a poussé, sans crier. Il tourne. [pause]</t>
+          <t>Le &lt;emphasis&gt;vent&lt;/emphasis&gt;, d'abord. J'ouvre un peu, à votre hauteur. Aniss attend, Mila tient le jaune. Le fil prend le vent de la porte. Une pale part, sans un mot. Ça tient ! La goutte de cire rouge file dans le courant, ronde. Le fil attend, autour du bâton. La porte a donné le courant. Aniss a poussé, sans crier. Le vent. [pause]</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -11195,7 +11195,7 @@
 narrateur|Le fil attend, autour du bâton.
 papa|La porte a donné le courant.
 maman|Aniss a poussé, sans crier.
-enfant-m|Il tourne.</t>
+enfant-m|Le vent.</t>
         </is>
       </c>
       <c r="AX54" t="inlineStr">
@@ -11227,17 +11227,17 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Le jaune rejoint la grille, tout sec. On a trouvé, Aniss. Le vent n'a pas glissé. Le porche a failli manger le vent. Entrez, le seuil est sec. Le fil pend, un peu humide, contre le fer. Un rai rouge s'allonge sur le bitume, puis s'arrête. Le vent de la porte lèche la goutte de cire rouge.</t>
+          <t>Le jaune rejoint la grille, tout sec. On a trouvé, Aniss. Le vent n'a pas glissé. Le fil a failli rester sans air. Entrez, le seuil est sec. Le fil pend, un peu humide, contre le fer. Un fil beige tremble, puis se tait. Le vent de la porte lèche la goutte de cire rouge.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jaune rejoint la grille, tout sec. On a trouvé, Aniss. Le vent n'a pas glissé. Le porche a failli manger le vent. Entrez, le seuil est sec. Le fil pend, un peu humide, contre le fer. Un rai rouge s'allonge sur le bitume, puis s'arrête. Le vent de la porte lèche la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jaune rejoint la grille, tout sec. On a trouvé, Aniss. Le vent n'a pas glissé. Le fil a failli rester sans air. Entrez, le seuil est sec. Le fil pend, un peu humide, contre le fer. Un fil beige tremble, puis se tait. Le vent de la porte lèche la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jaune rejoint la grille, tout sec. On a trouvé, Aniss. Le vent n'a pas glissé. Le porche a failli manger le vent. Entrez, le seuil est sec. Le fil pend, un peu humide, contre le fer. Un rai rouge s'allonge sur le bitume, puis s'arrête. Le vent de la porte lèche la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jaune rejoint la grille, tout sec. On a trouvé, Aniss. Le vent n'a pas glissé. Le fil a failli rester sans air. Entrez, le seuil est sec. Le fil pend, un peu humide, contre le fer. Un fil beige tremble, puis se tait. Le vent de la porte lèche la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -11378,10 +11378,10 @@
           <t>narrateur|Le jaune rejoint la grille, tout sec.
 copine|On a trouvé, Aniss.
 papa|Le vent n'a pas glissé.
-narrateur|Le porche a failli manger le vent.
+narrateur|Le fil a failli rester sans air.
 maman|Entrez, le seuil est sec.
 narrateur|Le fil pend, un peu humide, contre le fer.
-narrateur|Un rai rouge s'allonge sur le bitume, puis s'arrête.
+narrateur|Un fil beige tremble, puis se tait.
 narrateur|Le vent de la porte lèche la goutte de cire rouge.</t>
         </is>
       </c>
@@ -11414,17 +11414,17 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Mila. Aniss pointe la marche, du doigt. Mila attend, puis ouvre les mains. Le fil pose le papier sur la marche. Le courant du seuil pousse, tout net. Je le tiens. La goutte de cire rouge prend l'air, sur la marche. Le fil attend, autour du bâton. Le porche garde son ombre, plus loin. Tes mains ont guidé le moulin. Il tourne.</t>
+          <t>Mila. Aniss pointe la marche, du doigt. Mila attend, puis ouvre les mains. Le fil pose le papier sur la marche. Le courant du seuil pousse, tout net. Je le tiens. La goutte de cire rouge prend l'air, sur la marche. Le fil attend, autour du bâton. Le porche garde son ombre, plus loin. Tes mains ont guidé le moulin. La marche.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila. Aniss pointe la &lt;emphasis level="moderate"&gt;marche&lt;/emphasis&gt;, du doigt. Mila attend, puis ouvre les mains. Le fil pose le papier sur la marche. Le courant du seuil pousse, tout net. Je le tiens. La goutte de cire rouge prend l'air, sur la marche. Le fil attend, autour du bâton. Le porche garde son ombre, plus loin. Tes mains ont guidé le moulin. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila. Aniss pointe la &lt;emphasis level="moderate"&gt;marche&lt;/emphasis&gt;, du doigt. Mila attend, puis ouvre les mains. Le fil pose le papier sur la marche. Le courant du seuil pousse, tout net. Je le tiens. La goutte de cire rouge prend l'air, sur la marche. Le fil attend, autour du bâton. Le porche garde son ombre, plus loin. Tes mains ont guidé le moulin. La marche.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Mila. Aniss pointe la &lt;emphasis&gt;marche&lt;/emphasis&gt;, du doigt. Mila attend, puis ouvre les mains. Le fil pose le papier sur la marche. Le courant du seuil pousse, tout net. Je le tiens. La goutte de cire rouge prend l'air, sur la marche. Le fil attend, autour du bâton. Le porche garde son ombre, plus loin. Tes mains ont guidé le moulin. Il tourne. [pause]</t>
+          <t>Mila. Aniss pointe la &lt;emphasis&gt;marche&lt;/emphasis&gt;, du doigt. Mila attend, puis ouvre les mains. Le fil pose le papier sur la marche. Le courant du seuil pousse, tout net. Je le tiens. La goutte de cire rouge prend l'air, sur la marche. Le fil attend, autour du bâton. Le porche garde son ombre, plus loin. Tes mains ont guidé le moulin. La marche. [pause]</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -11568,7 +11568,7 @@
 narrateur|Le fil attend, autour du bâton.
 maman|Le porche garde son ombre, plus loin.
 papa|Tes mains ont guidé le moulin.
-enfant-m|Il tourne.</t>
+enfant-m|La marche.</t>
         </is>
       </c>
       <c r="AX56" t="inlineStr">
@@ -11600,17 +11600,17 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Les mains de Mila laissent le jaune au fer. On l'a tenu, tous les deux. Le porche est resté à sa place. Le porche a failli manger le vent. Essuie tes chaussures, Aniss. Le fil pend, un peu humide, contre le fer. Au muret, ça sent la cire, tiède. La marche tient la goutte de cire rouge, droite.</t>
+          <t>Les mains de Mila laissent le jaune au fer. On l'a tenu, tous les deux. Le porche est resté à sa place. Le fil a failli rester sans air. Essuie tes chaussures, Aniss. Le fil pend, un peu humide, contre le fer. Une pale sèche, contre le fer. La marche tient la goutte de cire rouge, droite.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les mains de Mila laissent le jaune au fer. On l'a tenu, tous les deux. Le porche est resté à sa place. Le porche a failli manger le vent. Essuie tes chaussures, Aniss. Le fil pend, un peu humide, contre le fer. Au muret, ça sent la cire, tiède. La marche tient la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;, droite.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les mains de Mila laissent le jaune au fer. On l'a tenu, tous les deux. Le porche est resté à sa place. Le fil a failli rester sans air. Essuie tes chaussures, Aniss. Le fil pend, un peu humide, contre le fer. Une pale sèche, contre le fer. La marche tient la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;, droite.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les mains de Mila laissent le jaune au fer. On l'a tenu, tous les deux. Le porche est resté à sa place. Le porche a failli manger le vent. Essuie tes chaussures, Aniss. Le fil pend, un peu humide, contre le fer. Au muret, ça sent la cire, tiède. La marche tient la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;, droite.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les mains de Mila laissent le jaune au fer. On l'a tenu, tous les deux. Le porche est resté à sa place. Le fil a failli rester sans air. Essuie tes chaussures, Aniss. Le fil pend, un peu humide, contre le fer. Une pale sèche, contre le fer. La marche tient la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;, droite.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -11751,10 +11751,10 @@
           <t>narrateur|Les mains de Mila laissent le jaune au fer.
 copine|On l'a tenu, tous les deux.
 papa|Le porche est resté à sa place.
-narrateur|Le porche a failli manger le vent.
+narrateur|Le fil a failli rester sans air.
 maman|Essuie tes chaussures, Aniss.
 narrateur|Le fil pend, un peu humide, contre le fer.
-narrateur|Au muret, ça sent la cire, tiède.
+narrateur|Une pale sèche, contre le fer.
 narrateur|La marche tient la goutte de cire rouge, droite.</t>
         </is>
       </c>
@@ -11787,17 +11787,17 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Le nœud, Aniss. Aniss pointe le crochet du porche, du doigt. Mila attend, puis suit le doigt. Le fil serre le nœud, tout droit. Le jaune se tient, hors du mur. Il évite le mur. La goutte de cire rouge veille derrière le nœud. Le fil attend, autour du bâton. Le nœud a montré la route. Vos pieds restent au sec, aussi. Il tourne.</t>
+          <t>Le nœud, Aniss. Aniss pointe le crochet du porche, du doigt. Mila attend, puis suit le doigt. Le fil serre le nœud, tout droit. Le jaune se tient, hors du mur. Il évite le mur. La goutte de cire rouge veille derrière le nœud. Le fil attend, autour du bâton. Le nœud a montré la route. Vos pieds restent au sec, aussi. Le nœud.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;nœud&lt;/emphasis&gt;, Aniss. Aniss pointe le crochet du porche, du doigt. Mila attend, puis suit le doigt. Le fil serre le nœud, tout droit. Le jaune se tient, hors du mur. Il évite le mur. La goutte de cire rouge veille derrière le nœud. Le fil attend, autour du bâton. Le nœud a montré la route. Vos pieds restent au sec, aussi. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;nœud&lt;/emphasis&gt;, Aniss. Aniss pointe le crochet du porche, du doigt. Mila attend, puis suit le doigt. Le fil serre le nœud, tout droit. Le jaune se tient, hors du mur. Il évite le mur. La goutte de cire rouge veille derrière le nœud. Le fil attend, autour du bâton. Le nœud a montré la route. Vos pieds restent au sec, aussi. Le nœud.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;nœud&lt;/emphasis&gt;, Aniss. Aniss pointe le crochet du porche, du doigt. Mila attend, puis suit le doigt. Le fil serre le nœud, tout droit. Le jaune se tient, hors du mur. Il évite le mur. La goutte de cire rouge veille derrière le nœud. Le fil attend, autour du bâton. Le nœud a montré la route. Vos pieds restent au sec, aussi. Il tourne. [pause]</t>
+          <t>Le &lt;emphasis&gt;nœud&lt;/emphasis&gt;, Aniss. Aniss pointe le crochet du porche, du doigt. Mila attend, puis suit le doigt. Le fil serre le nœud, tout droit. Le jaune se tient, hors du mur. Il évite le mur. La goutte de cire rouge veille derrière le nœud. Le fil attend, autour du bâton. Le nœud a montré la route. Vos pieds restent au sec, aussi. Le nœud. [pause]</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -11941,7 +11941,7 @@
 narrateur|Le fil attend, autour du bâton.
 papa|Le nœud a montré la route.
 maman|Vos pieds restent au sec, aussi.
-enfant-m|Il tourne.</t>
+enfant-m|Le nœud.</t>
         </is>
       </c>
       <c r="AX58" t="inlineStr">
@@ -11973,17 +11973,17 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Le jaune suit le nœud, jusqu'à la grille. L'ombre était douce. Le nœud a tenu, tout droit. Le porche a failli manger le vent. Le porche n'a plus rien à dire. Le fil pend, un peu humide, contre le fer. Au loin, le bus se tait. Le nœud serre près de la goutte de cire rouge.</t>
+          <t>Le jaune suit le nœud, jusqu'à la grille. L'ombre était douce. Le nœud a tenu, tout droit. Le fil a failli rester sans air. Le porche n'a plus rien à dire. Le fil pend, un peu humide, contre le fer. Sur le bitume, une trace d'eau, mince. Le nœud serre près de la goutte de cire rouge.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jaune suit le nœud, jusqu'à la grille. L'ombre était douce. Le nœud a tenu, tout droit. Le porche a failli manger le vent. Le porche n'a plus rien à dire. Le fil pend, un peu humide, contre le fer. Au loin, le bus se tait. Le nœud serre près de la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jaune suit le nœud, jusqu'à la grille. L'ombre était douce. Le nœud a tenu, tout droit. Le fil a failli rester sans air. Le porche n'a plus rien à dire. Le fil pend, un peu humide, contre le fer. Sur le bitume, une trace d'eau, mince. Le nœud serre près de la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jaune suit le nœud, jusqu'à la grille. L'ombre était douce. Le nœud a tenu, tout droit. Le porche a failli manger le vent. Le porche n'a plus rien à dire. Le fil pend, un peu humide, contre le fer. Au loin, le bus se tait. Le nœud serre près de la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jaune suit le nœud, jusqu'à la grille. L'ombre était douce. Le nœud a tenu, tout droit. Le fil a failli rester sans air. Le porche n'a plus rien à dire. Le fil pend, un peu humide, contre le fer. Sur le bitume, une trace d'eau, mince. Le nœud serre près de la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -12124,10 +12124,10 @@
           <t>narrateur|Le jaune suit le nœud, jusqu'à la grille.
 copine|L'ombre était douce.
 papa|Le nœud a tenu, tout droit.
-narrateur|Le porche a failli manger le vent.
+narrateur|Le fil a failli rester sans air.
 maman|Le porche n'a plus rien à dire.
 narrateur|Le fil pend, un peu humide, contre le fer.
-narrateur|Au loin, le bus se tait.
+narrateur|Sur le bitume, une trace d'eau, mince.
 narrateur|Le nœud serre près de la goutte de cire rouge.</t>
         </is>
       </c>
@@ -12918,17 +12918,17 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Le caillou reste coincé, trop large pour le fer. La grille serre trop, juste à hauteur d'Aniss. Force, Aniss ! Aniss montre un écart plus bas, du doigt. La pierre cogne, puis recule. Dis-moi où ! Aniss secoue la tête, tout petit. On ne fonce pas. Mila se tait, et son silence compte. Il montre, avec le doigt. Le crochet du loquet brille un peu. La goutte de cire rouge s'est cachée derrière un barreau. Vous faites comment, tous les deux ?</t>
+          <t>Le caillou reste coincé, trop large pour le fer. La pierre cogne un barreau, puis recule. Force, Aniss ! Aniss pose la pierre au pied de la grille. Il la fait rouler, le long du bas. Dis pierre ! Aniss appuie sur le caillou, tout petit. Elle passe là. Mila se tait, les lèvres fermées. La pierre a cherché l'écart. Le crochet du loquet brille un peu. La goutte de cire rouge s'est cachée derrière un barreau. Vous faites comment, tous les deux ?</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le caillou reste coincé, trop large pour le fer. La grille serre trop, juste à hauteur d'Aniss. Force, Aniss ! Aniss montre un écart plus bas, du doigt. La pierre cogne, puis recule. Dis-moi où ! Aniss secoue la tête, tout petit. On ne fonce pas. Mila se tait, et son silence compte. Il montre, avec le doigt. Le crochet du loquet brille un peu. La &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; s'est cachée derrière un barreau. Vous faites comment, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le caillou reste coincé, trop large pour le fer. La pierre cogne un barreau, puis recule. Force, Aniss ! Aniss pose la pierre au pied de la grille. Il la fait rouler, le long du bas. Dis pierre ! Aniss appuie sur le caillou, tout petit. Elle passe là. Mila se tait, les lèvres fermées. La pierre a cherché l'écart. Le crochet du loquet brille un peu. La &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; s'est cachée derrière un barreau. Vous faites comment, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Le caillou reste coincé, trop large pour le fer. La grille serre trop, juste à hauteur d'Aniss. Force, Aniss ! Aniss montre un écart plus bas, du doigt. La pierre cogne, puis recule. Dis-moi où ! Aniss secoue la tête, tout petit. On ne fonce pas. Mila se tait, et son silence compte. Il montre, avec le doigt. Le crochet du loquet brille un peu. La &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; s'est cachée derrière un barreau. Vous faites comment, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Le caillou reste coincé, trop large pour le fer. La pierre cogne un barreau, puis recule. Force, Aniss ! Aniss pose la pierre au pied de la grille. Il la fait rouler, le long du bas. Dis pierre ! Aniss appuie sur le caillou, tout petit. Elle passe là. Mila se tait, les lèvres fermées. La pierre a cherché l'écart. Le crochet du loquet brille un peu. La &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; s'est cachée derrière un barreau. Vous faites comment, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr"/>
@@ -13067,15 +13067,15 @@
       <c r="AW64" t="inlineStr">
         <is>
           <t>narrateur|Le caillou reste coincé, trop large pour le fer.
-narrateur|La grille serre trop, juste à hauteur d'Aniss.
+narrateur|La pierre cogne un barreau, puis recule.
 copine|Force, Aniss !
-narrateur|Aniss montre un écart plus bas, du doigt.
-narrateur|La pierre cogne, puis recule.
-copine|Dis-moi où !
-narrateur|Aniss secoue la tête, tout petit.
-enfant-m|On ne fonce pas.
-narrateur|Mila se tait, et son silence compte.
-maman|Il montre, avec le doigt.
+narrateur|Aniss pose la pierre au pied de la grille.
+narrateur|Il la fait rouler, le long du bas.
+copine|Dis pierre !
+narrateur|Aniss appuie sur le caillou, tout petit.
+enfant-m|Elle passe là.
+narrateur|Mila se tait, les lèvres fermées.
+maman|La pierre a cherché l'écart.
 papa|Le crochet du loquet brille un peu.
 narrateur|La goutte de cire rouge s'est cachée derrière un barreau.
 papa|Vous faites comment, tous les deux ?</t>
@@ -13307,17 +13307,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>On attend. Aniss cherche l'écart du bas, sans presser. Mila suit le doigt, enfin, un peu. Le caillou reste bas, près du bitume. Aniss glisse le bâton, sans un mot. Le fer fait toc, plus large. Toc. La goutte de cire rouge revoit le vent, ronde. Le caillou attend, contre le papier. Le bas laisse un vrai passage. Il tourne.</t>
+          <t>On attend. Aniss cherche l'écart du bas, sans presser. Mila suit le doigt, enfin, un peu. Le caillou reste bas, près du bitume. Aniss glisse le bâton, sans un mot. Le fer fait toc, plus large. Toc. La goutte de cire rouge revoit le vent, ronde. Le caillou attend, contre le papier. Le bas laisse un vrai passage. En bas.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend. Aniss cherche l'écart du &lt;emphasis level="moderate"&gt;bas&lt;/emphasis&gt;, sans presser. Mila suit le doigt, enfin, un peu. Le caillou reste bas, près du bitume. Aniss glisse le bâton, sans un mot. Le fer fait toc, plus large. Toc. La goutte de cire rouge revoit le vent, ronde. Le caillou attend, contre le papier. Le bas laisse un vrai passage. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend. Aniss cherche l'écart du &lt;emphasis level="moderate"&gt;bas&lt;/emphasis&gt;, sans presser. Mila suit le doigt, enfin, un peu. Le caillou reste bas, près du bitume. Aniss glisse le bâton, sans un mot. Le fer fait toc, plus large. Toc. La goutte de cire rouge revoit le vent, ronde. Le caillou attend, contre le papier. Le bas laisse un vrai passage. En bas.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>On attend. Aniss cherche l'écart du &lt;emphasis&gt;bas&lt;/emphasis&gt;, sans presser. Mila suit le doigt, enfin, un peu. Le caillou reste bas, près du bitume. Aniss glisse le bâton, sans un mot. Le fer fait toc, plus large. Toc. La goutte de cire rouge revoit le vent, ronde. Le caillou attend, contre le papier. Le bas laisse un vrai passage. Il tourne. [pause]</t>
+          <t>On attend. Aniss cherche l'écart du &lt;emphasis&gt;bas&lt;/emphasis&gt;, sans presser. Mila suit le doigt, enfin, un peu. Le caillou reste bas, près du bitume. Aniss glisse le bâton, sans un mot. Le fer fait toc, plus large. Toc. La goutte de cire rouge revoit le vent, ronde. Le caillou attend, contre le papier. Le bas laisse un vrai passage. En bas. [pause]</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -13461,7 +13461,7 @@
 narrateur|La goutte de cire rouge revoit le vent, ronde.
 narrateur|Le caillou attend, contre le papier.
 papa|Le bas laisse un vrai passage.
-enfant-m|Il tourne.</t>
+enfant-m|En bas.</t>
         </is>
       </c>
       <c r="AX66" t="inlineStr">
@@ -13493,17 +13493,17 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Le moulin pose une pale sur le fer. Tourne. Il est arrivé. Les barreaux ont failli garder le papier. Le bas a laissé le passage. Le caillou reste tiède, contre le barreau. Un rai rouge s'allonge sur le bitume, puis s'arrête. Le caillou cale la goutte de cire rouge au bas.</t>
+          <t>Le moulin pose une pale sur le fer. Tourne. Il est arrivé. Le caillou a failli coincer le bas. Le bas a laissé le passage. Le caillou reste tiède, contre le barreau. La pierre reste tiède, dans la paume. Le caillou cale la goutte de cire rouge au bas.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le moulin pose une pale sur le fer. Tourne. Il est arrivé. Les barreaux ont failli garder le papier. Le bas a laissé le passage. Le caillou reste tiède, contre le barreau. Un rai rouge s'allonge sur le bitume, puis s'arrête. Le caillou cale la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; au bas.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le moulin pose une pale sur le fer. Tourne. Il est arrivé. Le caillou a failli coincer le bas. Le bas a laissé le passage. Le caillou reste tiède, contre le barreau. La pierre reste tiède, dans la paume. Le caillou cale la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; au bas.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le moulin pose une pale sur le fer. Tourne. Il est arrivé. Les barreaux ont failli garder le papier. Le bas a laissé le passage. Le caillou reste tiède, contre le barreau. Un rai rouge s'allonge sur le bitume, puis s'arrête. Le caillou cale la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; au bas.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le moulin pose une pale sur le fer. Tourne. Il est arrivé. Le caillou a failli coincer le bas. Le bas a laissé le passage. Le caillou reste tiède, contre le barreau. La pierre reste tiède, dans la paume. Le caillou cale la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; au bas.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -13644,10 +13644,10 @@
           <t>narrateur|Le moulin pose une pale sur le fer.
 enfant-m|Tourne.
 copine|Il est arrivé.
-narrateur|Les barreaux ont failli garder le papier.
+narrateur|Le caillou a failli coincer le bas.
 papa|Le bas a laissé le passage.
 narrateur|Le caillou reste tiède, contre le barreau.
-narrateur|Un rai rouge s'allonge sur le bitume, puis s'arrête.
+narrateur|La pierre reste tiède, dans la paume.
 narrateur|Le caillou cale la goutte de cire rouge au bas.</t>
         </is>
       </c>
@@ -13680,17 +13680,17 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Pour toi. Mila ouvre les deux mains, tout près. Aniss pose le jaune contre ses paumes. Le caillou suit le papier vers Mila. Mila vise l'écart, Aniss pousse le bâton. Il passe ! La goutte de cire rouge échappe au fer, ronde. Le caillou attend, contre le papier. Tes mains ont trouvé le fer. Il l'a tendu, d'abord. Il tourne.</t>
+          <t>Pour toi. Mila ouvre les deux mains, tout près. Aniss pose le jaune contre ses paumes. Le caillou suit le papier vers Mila. Mila vise l'écart, Aniss pousse le bâton. Il passe ! La goutte de cire rouge échappe au fer, ronde. Le caillou attend, contre le papier. Tes mains ont trouvé le fer. Il l'a tendu, d'abord. Tes mains.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Pour toi. Mila ouvre les deux &lt;emphasis level="moderate"&gt;mains&lt;/emphasis&gt;, tout près. Aniss pose le jaune contre ses paumes. Le caillou suit le papier vers Mila. Mila vise l'écart, Aniss pousse le bâton. Il passe ! La goutte de cire rouge échappe au fer, ronde. Le caillou attend, contre le papier. Tes mains ont trouvé le fer. Il l'a tendu, d'abord. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Pour toi. Mila ouvre les deux &lt;emphasis level="moderate"&gt;mains&lt;/emphasis&gt;, tout près. Aniss pose le jaune contre ses paumes. Le caillou suit le papier vers Mila. Mila vise l'écart, Aniss pousse le bâton. Il passe ! La goutte de cire rouge échappe au fer, ronde. Le caillou attend, contre le papier. Tes mains ont trouvé le fer. Il l'a tendu, d'abord. Tes mains.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Pour toi. Mila ouvre les deux &lt;emphasis&gt;mains&lt;/emphasis&gt;, tout près. Aniss pose le jaune contre ses paumes. Le caillou suit le papier vers Mila. Mila vise l'écart, Aniss pousse le bâton. Il passe ! La goutte de cire rouge échappe au fer, ronde. Le caillou attend, contre le papier. Tes mains ont trouvé le fer. Il l'a tendu, d'abord. Il tourne. [pause]</t>
+          <t>Pour toi. Mila ouvre les deux &lt;emphasis&gt;mains&lt;/emphasis&gt;, tout près. Aniss pose le jaune contre ses paumes. Le caillou suit le papier vers Mila. Mila vise l'écart, Aniss pousse le bâton. Il passe ! La goutte de cire rouge échappe au fer, ronde. Le caillou attend, contre le papier. Tes mains ont trouvé le fer. Il l'a tendu, d'abord. Tes mains. [pause]</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -13834,7 +13834,7 @@
 narrateur|Le caillou attend, contre le papier.
 maman|Tes mains ont trouvé le fer.
 papa|Il l'a tendu, d'abord.
-enfant-m|Il tourne.</t>
+enfant-m|Tes mains.</t>
         </is>
       </c>
       <c r="AX68" t="inlineStr">
@@ -13866,17 +13866,17 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Le jaune s'est glissé jusqu'au barreau. Aniss l'a tendu, tout seul. Tu as tendu, d'abord. Les barreaux ont failli garder le papier. Venez, le moulin est près de la grille. Le caillou reste tiède, contre le barreau. Au muret, ça sent la cire, tiède. La pierre suit la goutte de cire rouge vers Mila.</t>
+          <t>Le jaune s'est glissé jusqu'au barreau. Aniss l'a tendu, tout seul. Tu as tendu, d'abord. Le caillou a failli coincer le bas. Venez, le moulin est près de la grille. Le caillou reste tiède, contre le barreau. Un toc de fer s'éteint, tout près. La pierre suit la goutte de cire rouge vers Mila.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jaune s'est glissé jusqu'au barreau. Aniss l'a tendu, tout seul. Tu as tendu, d'abord. Les barreaux ont failli garder le papier. Venez, le moulin est près de la grille. Le caillou reste tiède, contre le barreau. Au muret, ça sent la cire, tiède. La pierre suit la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; vers Mila.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jaune s'est glissé jusqu'au barreau. Aniss l'a tendu, tout seul. Tu as tendu, d'abord. Le caillou a failli coincer le bas. Venez, le moulin est près de la grille. Le caillou reste tiède, contre le barreau. Un toc de fer s'éteint, tout près. La pierre suit la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; vers Mila.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jaune s'est glissé jusqu'au barreau. Aniss l'a tendu, tout seul. Tu as tendu, d'abord. Les barreaux ont failli garder le papier. Venez, le moulin est près de la grille. Le caillou reste tiède, contre le barreau. Au muret, ça sent la cire, tiède. La pierre suit la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; vers Mila.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jaune s'est glissé jusqu'au barreau. Aniss l'a tendu, tout seul. Tu as tendu, d'abord. Le caillou a failli coincer le bas. Venez, le moulin est près de la grille. Le caillou reste tiède, contre le barreau. Un toc de fer s'éteint, tout près. La pierre suit la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; vers Mila.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -14017,10 +14017,10 @@
           <t>narrateur|Le jaune s'est glissé jusqu'au barreau.
 copine|Aniss l'a tendu, tout seul.
 papa|Tu as tendu, d'abord.
-narrateur|Les barreaux ont failli garder le papier.
+narrateur|Le caillou a failli coincer le bas.
 maman|Venez, le moulin est près de la grille.
 narrateur|Le caillou reste tiède, contre le barreau.
-narrateur|Au muret, ça sent la cire, tiède.
+narrateur|Un toc de fer s'éteint, tout près.
 narrateur|La pierre suit la goutte de cire rouge vers Mila.</t>
         </is>
       </c>
@@ -14053,17 +14053,17 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Le crochet, Aniss. Aniss lève le jaune, sans un mot. Mila attend, puis suit sa main. Le caillou cale le crochet du loquet. Une pale racle le fer, puis se libère. Il tient. La goutte de cire rouge reprend le rai, petite. Le caillou attend, contre le papier. Le loquet a gardé le papier. Les barreaux peuvent dormir, plus loin. Il tourne.</t>
+          <t>Le crochet, Aniss. Aniss lève le jaune, sans un mot. Mila attend, puis suit sa main. Le caillou cale le crochet du loquet. Une pale racle le fer, puis se libère. Il tient. La goutte de cire rouge reprend le rai, petite. Le caillou attend, contre le papier. Le loquet a gardé le papier. Les barreaux peuvent dormir, plus loin. Au crochet.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;crochet&lt;/emphasis&gt;, Aniss. Aniss lève le jaune, sans un mot. Mila attend, puis suit sa main. Le caillou cale le crochet du loquet. Une pale racle le fer, puis se libère. Il tient. La goutte de cire rouge reprend le rai, petite. Le caillou attend, contre le papier. Le loquet a gardé le papier. Les barreaux peuvent dormir, plus loin. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;crochet&lt;/emphasis&gt;, Aniss. Aniss lève le jaune, sans un mot. Mila attend, puis suit sa main. Le caillou cale le crochet du loquet. Une pale racle le fer, puis se libère. Il tient. La goutte de cire rouge reprend le rai, petite. Le caillou attend, contre le papier. Le loquet a gardé le papier. Les barreaux peuvent dormir, plus loin. Au crochet.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;crochet&lt;/emphasis&gt;, Aniss. Aniss lève le jaune, sans un mot. Mila attend, puis suit sa main. Le caillou cale le crochet du loquet. Une pale racle le fer, puis se libère. Il tient. La goutte de cire rouge reprend le rai, petite. Le caillou attend, contre le papier. Le loquet a gardé le papier. Les barreaux peuvent dormir, plus loin. Il tourne. [pause]</t>
+          <t>Le &lt;emphasis&gt;crochet&lt;/emphasis&gt;, Aniss. Aniss lève le jaune, sans un mot. Mila attend, puis suit sa main. Le caillou cale le crochet du loquet. Une pale racle le fer, puis se libère. Il tient. La goutte de cire rouge reprend le rai, petite. Le caillou attend, contre le papier. Le loquet a gardé le papier. Les barreaux peuvent dormir, plus loin. Au crochet. [pause]</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
@@ -14207,7 +14207,7 @@
 narrateur|Le caillou attend, contre le papier.
 papa|Le loquet a gardé le papier.
 maman|Les barreaux peuvent dormir, plus loin.
-enfant-m|Il tourne.</t>
+enfant-m|Au crochet.</t>
         </is>
       </c>
       <c r="AX70" t="inlineStr">
@@ -14239,17 +14239,17 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Le jaune pend au crochet, tout droit. On a posé le moulin. Le crochet a tenu, tout droit. Les barreaux ont failli garder le papier. Essuyez vos mains, tout près. Le caillou reste tiède, contre le barreau. Au loin, le bus se tait. Le crochet pince la goutte de cire rouge, sans la casser.</t>
+          <t>Le jaune pend au crochet, tout droit. On a posé le moulin. Le crochet a tenu, tout droit. Le caillou a failli coincer le bas. Essuyez vos mains, tout près. Le caillou reste tiède, contre le barreau. L'ombre du porche recule, un peu. Le crochet pince la goutte de cire rouge, sans la casser.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jaune pend au crochet, tout droit. On a posé le moulin. Le crochet a tenu, tout droit. Les barreaux ont failli garder le papier. Essuyez vos mains, tout près. Le caillou reste tiède, contre le barreau. Au loin, le bus se tait. Le crochet pince la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;, sans la casser.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jaune pend au crochet, tout droit. On a posé le moulin. Le crochet a tenu, tout droit. Le caillou a failli coincer le bas. Essuyez vos mains, tout près. Le caillou reste tiède, contre le barreau. L'ombre du porche recule, un peu. Le crochet pince la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;, sans la casser.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jaune pend au crochet, tout droit. On a posé le moulin. Le crochet a tenu, tout droit. Les barreaux ont failli garder le papier. Essuyez vos mains, tout près. Le caillou reste tiède, contre le barreau. Au loin, le bus se tait. Le crochet pince la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;, sans la casser.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jaune pend au crochet, tout droit. On a posé le moulin. Le crochet a tenu, tout droit. Le caillou a failli coincer le bas. Essuyez vos mains, tout près. Le caillou reste tiède, contre le barreau. L'ombre du porche recule, un peu. Le crochet pince la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;, sans la casser.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr"/>
@@ -14390,10 +14390,10 @@
           <t>narrateur|Le jaune pend au crochet, tout droit.
 copine|On a posé le moulin.
 papa|Le crochet a tenu, tout droit.
-narrateur|Les barreaux ont failli garder le papier.
+narrateur|Le caillou a failli coincer le bas.
 maman|Essuyez vos mains, tout près.
 narrateur|Le caillou reste tiède, contre le barreau.
-narrateur|Au loin, le bus se tait.
+narrateur|L'ombre du porche recule, un peu.
 narrateur|Le crochet pince la goutte de cire rouge, sans la casser.</t>
         </is>
       </c>
@@ -14426,17 +14426,17 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Le caillou glisse vers l'eau, trop vite. L'eau est trop grande. Une feuille jaune part, plus bas. Attrape la pierre ! Aniss recule le caillou, sans presser. L'eau frappe la dalle, puis rebondit. On ne fonce pas. Mila referme la bouche. Son silence compte, comme une réponse. La dalle tient le courant. On reste près du caniveau, tous les deux. La goutte de cire rouge s'est ternie, trop près de l'eau. Vous faites comment, tous les deux ?</t>
+          <t>Le caillou glisse vers l'eau, trop vite. L'eau est trop grande. La pierre veut partir avec la feuille jaune. Attrape la pierre ! Aniss cale le caillou contre la dalle. L'eau frappe, puis recule un peu. Elle reste là. Mila referme la bouche. Elle pose un genou, tout près d'Aniss. La dalle tient le courant. On reste près du caniveau, tous les deux. La goutte de cire rouge s'est ternie, trop près de l'eau. Vous faites comment, tous les deux ?</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le caillou glisse vers l'eau, trop vite. L'eau est trop grande. Une feuille jaune part, plus bas. Attrape la pierre ! Aniss recule le caillou, sans presser. L'eau frappe la dalle, puis rebondit. On ne fonce pas. Mila referme la bouche. Son silence compte, comme une réponse. La dalle tient le courant. On reste près du caniveau, tous les deux. La &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; s'est ternie, trop près de l'eau. Vous faites comment, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le caillou glisse vers l'eau, trop vite. L'eau est trop grande. La pierre veut partir avec la feuille jaune. Attrape la pierre ! Aniss cale le caillou contre la dalle. L'eau frappe, puis recule un peu. Elle reste là. Mila referme la bouche. Elle pose un genou, tout près d'Aniss. La dalle tient le courant. On reste près du caniveau, tous les deux. La &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; s'est ternie, trop près de l'eau. Vous faites comment, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Le caillou glisse vers l'eau, trop vite. L'eau est trop grande. Une feuille jaune part, plus bas. Attrape la pierre ! Aniss recule le caillou, sans presser. L'eau frappe la dalle, puis rebondit. On ne fonce pas. Mila referme la bouche. Son silence compte, comme une réponse. La dalle tient le courant. On reste près du caniveau, tous les deux. La &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; s'est ternie, trop près de l'eau. Vous faites comment, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Le caillou glisse vers l'eau, trop vite. L'eau est trop grande. La pierre veut partir avec la feuille jaune. Attrape la pierre ! Aniss cale le caillou contre la dalle. L'eau frappe, puis recule un peu. Elle reste là. Mila referme la bouche. Elle pose un genou, tout près d'Aniss. La dalle tient le courant. On reste près du caniveau, tous les deux. La &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; s'est ternie, trop près de l'eau. Vous faites comment, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
@@ -14576,13 +14576,13 @@
         <is>
           <t>narrateur|Le caillou glisse vers l'eau, trop vite.
 copine|L'eau est trop grande.
-narrateur|Une feuille jaune part, plus bas.
+narrateur|La pierre veut partir avec la feuille jaune.
 copine|Attrape la pierre !
-narrateur|Aniss recule le caillou, sans presser.
-narrateur|L'eau frappe la dalle, puis rebondit.
-enfant-m|On ne fonce pas.
+narrateur|Aniss cale le caillou contre la dalle.
+narrateur|L'eau frappe, puis recule un peu.
+enfant-m|Elle reste là.
 narrateur|Mila referme la bouche.
-narrateur|Son silence compte, comme une réponse.
+narrateur|Elle pose un genou, tout près d'Aniss.
 maman|La dalle tient le courant.
 papa|On reste près du caniveau, tous les deux.
 narrateur|La goutte de cire rouge s'est ternie, trop près de l'eau.
@@ -14815,17 +14815,17 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>On attend l'eau. Aniss s'assoit près du caniveau, sans presser. Mila s'assoit aussi, les genoux contre lui. Le caillou sèche contre la dalle. L'eau frappe, puis la feuille s'arrête. Maintenant. La goutte de cire rouge sèche, ronde, sur la dalle. Le caillou attend, contre le papier. La dalle a cassé le courant. Vous avez laissé l'eau finir. Il tourne.</t>
+          <t>On attend l'eau. Aniss s'assoit près du caniveau, sans presser. Mila s'assoit aussi, les genoux contre lui. Le caillou sèche contre la dalle. L'eau frappe, puis la feuille s'arrête. Maintenant. La goutte de cire rouge sèche, ronde, sur la dalle. Le caillou attend, contre le papier. La dalle a cassé le courant. Vous avez laissé l'eau finir. La dalle.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend l'eau. Aniss s'assoit près du caniveau, sans presser. Mila s'assoit aussi, les genoux contre lui. Le caillou sèche contre la &lt;emphasis level="moderate"&gt;dalle&lt;/emphasis&gt;. L'eau frappe, puis la feuille s'arrête. Maintenant. La goutte de cire rouge sèche, ronde, sur la dalle. Le caillou attend, contre le papier. La dalle a cassé le courant. Vous avez laissé l'eau finir. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend l'eau. Aniss s'assoit près du caniveau, sans presser. Mila s'assoit aussi, les genoux contre lui. Le caillou sèche contre la &lt;emphasis level="moderate"&gt;dalle&lt;/emphasis&gt;. L'eau frappe, puis la feuille s'arrête. Maintenant. La goutte de cire rouge sèche, ronde, sur la dalle. Le caillou attend, contre le papier. La dalle a cassé le courant. Vous avez laissé l'eau finir. La dalle.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>On attend l'eau. Aniss s'assoit près du caniveau, sans presser. Mila s'assoit aussi, les genoux contre lui. Le caillou sèche contre la &lt;emphasis&gt;dalle&lt;/emphasis&gt;. L'eau frappe, puis la feuille s'arrête. Maintenant. La goutte de cire rouge sèche, ronde, sur la dalle. Le caillou attend, contre le papier. La dalle a cassé le courant. Vous avez laissé l'eau finir. Il tourne. [pause]</t>
+          <t>On attend l'eau. Aniss s'assoit près du caniveau, sans presser. Mila s'assoit aussi, les genoux contre lui. Le caillou sèche contre la &lt;emphasis&gt;dalle&lt;/emphasis&gt;. L'eau frappe, puis la feuille s'arrête. Maintenant. La goutte de cire rouge sèche, ronde, sur la dalle. Le caillou attend, contre le papier. La dalle a cassé le courant. Vous avez laissé l'eau finir. La dalle. [pause]</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -14969,7 +14969,7 @@
 narrateur|Le caillou attend, contre le papier.
 papa|La dalle a cassé le courant.
 maman|Vous avez laissé l'eau finir.
-enfant-m|Il tourne.</t>
+enfant-m|La dalle.</t>
         </is>
       </c>
       <c r="AX74" t="inlineStr">
@@ -15001,17 +15001,17 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Le jaune rejoint la grille, un peu mouillé. On a attendu l'eau. Le caniveau n'a plus pris vos bras. L'eau a failli emporter la pale. Rentrez le fil, après la grille. Le caillou reste tiède, contre le barreau. Un rai rouge s'allonge sur le bitume, puis s'arrête. La dalle a séché la goutte de cire rouge.</t>
+          <t>Le jaune rejoint la grille, un peu mouillé. On a attendu l'eau. Le caniveau n'a plus pris vos bras. Le caillou a failli rouler au fond. Rentrez le fil, après la grille. Le caillou reste tiède, contre le barreau. La pierre reste tiède, dans la paume. La dalle a séché la goutte de cire rouge.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jaune rejoint la grille, un peu mouillé. On a attendu l'eau. Le caniveau n'a plus pris vos bras. L'eau a failli emporter la pale. Rentrez le fil, après la grille. Le caillou reste tiède, contre le barreau. Un rai rouge s'allonge sur le bitume, puis s'arrête. La dalle a séché la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jaune rejoint la grille, un peu mouillé. On a attendu l'eau. Le caniveau n'a plus pris vos bras. Le caillou a failli rouler au fond. Rentrez le fil, après la grille. Le caillou reste tiède, contre le barreau. La pierre reste tiède, dans la paume. La dalle a séché la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jaune rejoint la grille, un peu mouillé. On a attendu l'eau. Le caniveau n'a plus pris vos bras. L'eau a failli emporter la pale. Rentrez le fil, après la grille. Le caillou reste tiède, contre le barreau. Un rai rouge s'allonge sur le bitume, puis s'arrête. La dalle a séché la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jaune rejoint la grille, un peu mouillé. On a attendu l'eau. Le caniveau n'a plus pris vos bras. Le caillou a failli rouler au fond. Rentrez le fil, après la grille. Le caillou reste tiède, contre le barreau. La pierre reste tiède, dans la paume. La dalle a séché la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -15152,10 +15152,10 @@
           <t>narrateur|Le jaune rejoint la grille, un peu mouillé.
 copine|On a attendu l'eau.
 papa|Le caniveau n'a plus pris vos bras.
-narrateur|L'eau a failli emporter la pale.
+narrateur|Le caillou a failli rouler au fond.
 maman|Rentrez le fil, après la grille.
 narrateur|Le caillou reste tiède, contre le barreau.
-narrateur|Un rai rouge s'allonge sur le bitume, puis s'arrête.
+narrateur|La pierre reste tiède, dans la paume.
 narrateur|La dalle a séché la goutte de cire rouge.</t>
         </is>
       </c>
@@ -15188,17 +15188,17 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Tes mains, Aniss. Aniss tend le fil, tout près. Mila tire avec lui, sans presser. Le caillou guide le fil, tout droit. Le papier passe au-dessus de l'eau. On tient ensemble. La goutte de cire rouge tremble au bout du fil. Le caillou attend, contre le papier. Vos mains suffisent, toutes les deux. L'eau restera après. Il tourne.</t>
+          <t>Tes mains, Aniss. Aniss tend le fil, tout près. Mila tire avec lui, sans presser. Le caillou guide le fil, tout droit. Le papier passe au-dessus de l'eau. On tient ensemble. La goutte de cire rouge tremble au bout du fil. Le caillou attend, contre le papier. Vos mains suffisent, toutes les deux. L'eau restera après. On tient.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tes mains, Aniss. Aniss tend le &lt;emphasis level="moderate"&gt;fil&lt;/emphasis&gt;, tout près. Mila tire avec lui, sans presser. Le caillou guide le fil, tout droit. Le papier passe au-dessus de l'eau. On tient ensemble. La goutte de cire rouge tremble au bout du fil. Le caillou attend, contre le papier. Vos mains suffisent, toutes les deux. L'eau restera après. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tes mains, Aniss. Aniss tend le &lt;emphasis level="moderate"&gt;fil&lt;/emphasis&gt;, tout près. Mila tire avec lui, sans presser. Le caillou guide le fil, tout droit. Le papier passe au-dessus de l'eau. On tient ensemble. La goutte de cire rouge tremble au bout du fil. Le caillou attend, contre le papier. Vos mains suffisent, toutes les deux. L'eau restera après. On tient.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Tes mains, Aniss. Aniss tend le &lt;emphasis&gt;fil&lt;/emphasis&gt;, tout près. Mila tire avec lui, sans presser. Le caillou guide le fil, tout droit. Le papier passe au-dessus de l'eau. On tient ensemble. La goutte de cire rouge tremble au bout du fil. Le caillou attend, contre le papier. Vos mains suffisent, toutes les deux. L'eau restera après. Il tourne. [pause]</t>
+          <t>Tes mains, Aniss. Aniss tend le &lt;emphasis&gt;fil&lt;/emphasis&gt;, tout près. Mila tire avec lui, sans presser. Le caillou guide le fil, tout droit. Le papier passe au-dessus de l'eau. On tient ensemble. La goutte de cire rouge tremble au bout du fil. Le caillou attend, contre le papier. Vos mains suffisent, toutes les deux. L'eau restera après. On tient. [pause]</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -15342,7 +15342,7 @@
 narrateur|Le caillou attend, contre le papier.
 maman|Vos mains suffisent, toutes les deux.
 papa|L'eau restera après.
-enfant-m|Il tourne.</t>
+enfant-m|On tient.</t>
         </is>
       </c>
       <c r="AX76" t="inlineStr">
@@ -15374,17 +15374,17 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Le fil pose le moulin contre le fer. On tenait, tous les deux. Je remporte le fil, tout à l'heure. L'eau a failli emporter la pale. La grille vous attend. Le caillou reste tiède, contre le barreau. Au muret, ça sent la cire, tiède. Le caillou guide la goutte de cire rouge au-dessus de l'eau.</t>
+          <t>Le fil pose le moulin contre le fer. On tenait, tous les deux. Je remporte le fil, tout à l'heure. Le caillou a failli rouler au fond. La grille vous attend. Le caillou reste tiède, contre le barreau. Un toc de fer s'éteint, tout près. Le caillou guide la goutte de cire rouge au-dessus de l'eau.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le fil pose le moulin contre le fer. On tenait, tous les deux. Je remporte le fil, tout à l'heure. L'eau a failli emporter la pale. La grille vous attend. Le caillou reste tiède, contre le barreau. Au muret, ça sent la cire, tiède. Le caillou guide la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; au-dessus de l'eau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le fil pose le moulin contre le fer. On tenait, tous les deux. Je remporte le fil, tout à l'heure. Le caillou a failli rouler au fond. La grille vous attend. Le caillou reste tiède, contre le barreau. Un toc de fer s'éteint, tout près. Le caillou guide la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; au-dessus de l'eau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le fil pose le moulin contre le fer. On tenait, tous les deux. Je remporte le fil, tout à l'heure. L'eau a failli emporter la pale. La grille vous attend. Le caillou reste tiède, contre le barreau. Au muret, ça sent la cire, tiède. Le caillou guide la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; au-dessus de l'eau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le fil pose le moulin contre le fer. On tenait, tous les deux. Je remporte le fil, tout à l'heure. Le caillou a failli rouler au fond. La grille vous attend. Le caillou reste tiède, contre le barreau. Un toc de fer s'éteint, tout près. Le caillou guide la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; au-dessus de l'eau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr"/>
@@ -15525,10 +15525,10 @@
           <t>narrateur|Le fil pose le moulin contre le fer.
 copine|On tenait, tous les deux.
 papa|Je remporte le fil, tout à l'heure.
-narrateur|L'eau a failli emporter la pale.
+narrateur|Le caillou a failli rouler au fond.
 maman|La grille vous attend.
 narrateur|Le caillou reste tiède, contre le barreau.
-narrateur|Au muret, ça sent la cire, tiède.
+narrateur|Un toc de fer s'éteint, tout près.
 narrateur|Le caillou guide la goutte de cire rouge au-dessus de l'eau.</t>
         </is>
       </c>
@@ -15561,17 +15561,17 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Le bord, d'abord. Mila tend la pierre sèche vers Aniss. Aniss marche, sans un mot. Le caillou suit le bord sec. Une goutte rejoint le fond, puis se tait. C'est doux. La goutte de cire rouge reste au sec, sur le bord. Le caillou attend, contre le papier. L'eau garde son souffle, plus loin. Le bord a laissé le papier. Il tourne.</t>
+          <t>Le bord, d'abord. Mila tend la pierre sèche vers Aniss. Aniss marche, sans un mot. Le caillou suit le bord sec. Une goutte rejoint le fond, puis se tait. C'est doux. La goutte de cire rouge reste au sec, sur le bord. Le caillou attend, contre le papier. L'eau garde son souffle, plus loin. Le bord a laissé le papier. Au sec.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;bord&lt;/emphasis&gt;, d'abord. Mila tend la pierre sèche vers Aniss. Aniss marche, sans un mot. Le caillou suit le bord sec. Une goutte rejoint le fond, puis se tait. C'est doux. La goutte de cire rouge reste au sec, sur le bord. Le caillou attend, contre le papier. L'eau garde son souffle, plus loin. Le bord a laissé le papier. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;bord&lt;/emphasis&gt;, d'abord. Mila tend la pierre sèche vers Aniss. Aniss marche, sans un mot. Le caillou suit le bord sec. Une goutte rejoint le fond, puis se tait. C'est doux. La goutte de cire rouge reste au sec, sur le bord. Le caillou attend, contre le papier. L'eau garde son souffle, plus loin. Le bord a laissé le papier. Au sec.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;bord&lt;/emphasis&gt;, d'abord. Mila tend la pierre sèche vers Aniss. Aniss marche, sans un mot. Le caillou suit le bord sec. Une goutte rejoint le fond, puis se tait. C'est doux. La goutte de cire rouge reste au sec, sur le bord. Le caillou attend, contre le papier. L'eau garde son souffle, plus loin. Le bord a laissé le papier. Il tourne. [pause]</t>
+          <t>Le &lt;emphasis&gt;bord&lt;/emphasis&gt;, d'abord. Mila tend la pierre sèche vers Aniss. Aniss marche, sans un mot. Le caillou suit le bord sec. Une goutte rejoint le fond, puis se tait. C'est doux. La goutte de cire rouge reste au sec, sur le bord. Le caillou attend, contre le papier. L'eau garde son souffle, plus loin. Le bord a laissé le papier. Au sec. [pause]</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -15715,7 +15715,7 @@
 narrateur|Le caillou attend, contre le papier.
 maman|L'eau garde son souffle, plus loin.
 papa|Le bord a laissé le papier.
-enfant-m|Il tourne.</t>
+enfant-m|Au sec.</t>
         </is>
       </c>
       <c r="AX78" t="inlineStr">
@@ -15747,17 +15747,17 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Les mains d'Aniss laissent le jaune contre le fer. C'était plus facile, là. Tes bras ont guidé le moulin. L'eau a failli emporter la pale. Le barreau gardera son ombre. Le caillou reste tiède, contre le barreau. Au loin, le bus se tait. Le bord laisse la goutte de cire rouge au sec.</t>
+          <t>Les mains d'Aniss laissent le jaune contre le fer. C'était plus facile, là. Tes bras ont guidé le moulin. Le caillou a failli rouler au fond. Le barreau gardera son ombre. Le caillou reste tiède, contre le barreau. L'ombre du porche recule, un peu. Le bord laisse la goutte de cire rouge au sec.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les mains d'Aniss laissent le jaune contre le fer. C'était plus facile, là. Tes bras ont guidé le moulin. L'eau a failli emporter la pale. Le barreau gardera son ombre. Le caillou reste tiède, contre le barreau. Au loin, le bus se tait. Le bord laisse la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; au sec.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les mains d'Aniss laissent le jaune contre le fer. C'était plus facile, là. Tes bras ont guidé le moulin. Le caillou a failli rouler au fond. Le barreau gardera son ombre. Le caillou reste tiède, contre le barreau. L'ombre du porche recule, un peu. Le bord laisse la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; au sec.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les mains d'Aniss laissent le jaune contre le fer. C'était plus facile, là. Tes bras ont guidé le moulin. L'eau a failli emporter la pale. Le barreau gardera son ombre. Le caillou reste tiède, contre le barreau. Au loin, le bus se tait. Le bord laisse la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; au sec.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les mains d'Aniss laissent le jaune contre le fer. C'était plus facile, là. Tes bras ont guidé le moulin. Le caillou a failli rouler au fond. Le barreau gardera son ombre. Le caillou reste tiède, contre le barreau. L'ombre du porche recule, un peu. Le bord laisse la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; au sec.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -15898,10 +15898,10 @@
           <t>narrateur|Les mains d'Aniss laissent le jaune contre le fer.
 copine|C'était plus facile, là.
 papa|Tes bras ont guidé le moulin.
-narrateur|L'eau a failli emporter la pale.
+narrateur|Le caillou a failli rouler au fond.
 maman|Le barreau gardera son ombre.
 narrateur|Le caillou reste tiède, contre le barreau.
-narrateur|Au loin, le bus se tait.
+narrateur|L'ombre du porche recule, un peu.
 narrateur|Le bord laisse la goutte de cire rouge au sec.</t>
         </is>
       </c>
@@ -15934,17 +15934,17 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Le caillou reste lourd, sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis vent ! Aniss pointe la porte, du doigt. Le porche garde l'air, trop fermé. On ne fonce pas. Mila se tait, les joues gonflées. Son silence compte, comme une réponse. Tes yeux vont plus loin, Aniss. La marche du seuil est sèche. La goutte de cire rouge s'est éteinte, dans l'ombre. Vous faites comment, tous les deux ?</t>
+          <t>Le caillou reste lourd, sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis pierre ! Aniss pose le caillou sur la marche. Le papier ne bouge plus, trop bas. Plus haut. Mila se tait, les joues dégonflées. Elle pose les mains autour de la pierre. Tes yeux vont plus loin, Aniss. La marche du seuil est sèche. La goutte de cire rouge s'est éteinte, dans l'ombre. Vous faites comment, tous les deux ?</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le caillou reste lourd, sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis vent ! Aniss pointe la porte, du doigt. Le porche garde l'air, trop fermé. On ne fonce pas. Mila se tait, les joues gonflées. Son silence compte, comme une réponse. Tes yeux vont plus loin, Aniss. La marche du seuil est sèche. La &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; s'est éteinte, dans l'ombre. Vous faites comment, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Le caillou reste lourd, sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis pierre ! Aniss pose le caillou sur la marche. Le papier ne bouge plus, trop bas. Plus haut. Mila se tait, les joues dégonflées. Elle pose les mains autour de la pierre. Tes yeux vont plus loin, Aniss. La marche du seuil est sèche. La &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; s'est éteinte, dans l'ombre. Vous faites comment, tous les deux ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Le caillou reste lourd, sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis vent ! Aniss pointe la porte, du doigt. Le porche garde l'air, trop fermé. On ne fonce pas. Mila se tait, les joues gonflées. Son silence compte, comme une réponse. Tes yeux vont plus loin, Aniss. La marche du seuil est sèche. La &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; s'est éteinte, dans l'ombre. Vous faites comment, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Le caillou reste lourd, sous le porche. Ça ne tourne plus, Aniss ! Mila souffle trop vite, trop fort. Dis pierre ! Aniss pose le caillou sur la marche. Le papier ne bouge plus, trop bas. Plus haut. Mila se tait, les joues dégonflées. Elle pose les mains autour de la pierre. Tes yeux vont plus loin, Aniss. La marche du seuil est sèche. La &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; s'est éteinte, dans l'ombre. Vous faites comment, tous les deux ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
@@ -16085,12 +16085,12 @@
           <t>narrateur|Le caillou reste lourd, sous le porche.
 copine|Ça ne tourne plus, Aniss !
 narrateur|Mila souffle trop vite, trop fort.
-copine|Dis vent !
-narrateur|Aniss pointe la porte, du doigt.
-narrateur|Le porche garde l'air, trop fermé.
-enfant-m|On ne fonce pas.
-narrateur|Mila se tait, les joues gonflées.
-narrateur|Son silence compte, comme une réponse.
+copine|Dis pierre !
+narrateur|Aniss pose le caillou sur la marche.
+narrateur|Le papier ne bouge plus, trop bas.
+enfant-m|Plus haut.
+narrateur|Mila se tait, les joues dégonflées.
+narrateur|Elle pose les mains autour de la pierre.
 maman|Tes yeux vont plus loin, Aniss.
 papa|La marche du seuil est sèche.
 narrateur|La goutte de cire rouge s'est éteinte, dans l'ombre.
@@ -16323,17 +16323,17 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Le vent, d'abord. J'ouvre un peu, à votre hauteur. Aniss attend, Mila tient le jaune. Le caillou prend le vent de la porte. Une pale part, sans un mot. Ça tient ! La goutte de cire rouge file dans le courant, ronde. Le caillou attend, contre le papier. La porte a donné le courant. Aniss a poussé, sans crier. Il tourne.</t>
+          <t>Le vent, d'abord. J'ouvre un peu, à votre hauteur. Aniss attend, Mila tient le jaune. Le caillou prend le vent de la porte. Une pale part, sans un mot. Ça tient ! La goutte de cire rouge file dans le courant, ronde. Le caillou attend, contre le papier. La porte a donné le courant. Aniss a poussé, sans crier. Le vent.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;vent&lt;/emphasis&gt;, d'abord. J'ouvre un peu, à votre hauteur. Aniss attend, Mila tient le jaune. Le caillou prend le vent de la porte. Une pale part, sans un mot. Ça tient ! La goutte de cire rouge file dans le courant, ronde. Le caillou attend, contre le papier. La porte a donné le courant. Aniss a poussé, sans crier. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;vent&lt;/emphasis&gt;, d'abord. J'ouvre un peu, à votre hauteur. Aniss attend, Mila tient le jaune. Le caillou prend le vent de la porte. Une pale part, sans un mot. Ça tient ! La goutte de cire rouge file dans le courant, ronde. Le caillou attend, contre le papier. La porte a donné le courant. Aniss a poussé, sans crier. Le vent.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;vent&lt;/emphasis&gt;, d'abord. J'ouvre un peu, à votre hauteur. Aniss attend, Mila tient le jaune. Le caillou prend le vent de la porte. Une pale part, sans un mot. Ça tient ! La goutte de cire rouge file dans le courant, ronde. Le caillou attend, contre le papier. La porte a donné le courant. Aniss a poussé, sans crier. Il tourne. [pause]</t>
+          <t>Le &lt;emphasis&gt;vent&lt;/emphasis&gt;, d'abord. J'ouvre un peu, à votre hauteur. Aniss attend, Mila tient le jaune. Le caillou prend le vent de la porte. Une pale part, sans un mot. Ça tient ! La goutte de cire rouge file dans le courant, ronde. Le caillou attend, contre le papier. La porte a donné le courant. Aniss a poussé, sans crier. Le vent. [pause]</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
@@ -16477,7 +16477,7 @@
 narrateur|Le caillou attend, contre le papier.
 papa|La porte a donné le courant.
 maman|Aniss a poussé, sans crier.
-enfant-m|Il tourne.</t>
+enfant-m|Le vent.</t>
         </is>
       </c>
       <c r="AX82" t="inlineStr">
@@ -16509,17 +16509,17 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Le jaune rejoint la grille, tout sec. On a trouvé, Aniss. Le vent n'a pas glissé. Le porche a failli manger le vent. Entrez, le seuil est sec. Le caillou reste tiède, contre le barreau. Un rai rouge s'allonge sur le bitume, puis s'arrête. Le vent pousse la goutte de cire rouge, hors du mur.</t>
+          <t>Le jaune rejoint la grille, tout sec. On a trouvé, Aniss. Le vent n'a pas glissé. Le caillou a failli trop peser. Entrez, le seuil est sec. Le caillou reste tiède, contre le barreau. La pierre reste tiède, dans la paume. Le vent pousse la goutte de cire rouge, hors du mur.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jaune rejoint la grille, tout sec. On a trouvé, Aniss. Le vent n'a pas glissé. Le porche a failli manger le vent. Entrez, le seuil est sec. Le caillou reste tiède, contre le barreau. Un rai rouge s'allonge sur le bitume, puis s'arrête. Le vent pousse la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;, hors du mur.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jaune rejoint la grille, tout sec. On a trouvé, Aniss. Le vent n'a pas glissé. Le caillou a failli trop peser. Entrez, le seuil est sec. Le caillou reste tiède, contre le barreau. La pierre reste tiède, dans la paume. Le vent pousse la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt;, hors du mur.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jaune rejoint la grille, tout sec. On a trouvé, Aniss. Le vent n'a pas glissé. Le porche a failli manger le vent. Entrez, le seuil est sec. Le caillou reste tiède, contre le barreau. Un rai rouge s'allonge sur le bitume, puis s'arrête. Le vent pousse la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;, hors du mur.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jaune rejoint la grille, tout sec. On a trouvé, Aniss. Le vent n'a pas glissé. Le caillou a failli trop peser. Entrez, le seuil est sec. Le caillou reste tiède, contre le barreau. La pierre reste tiède, dans la paume. Le vent pousse la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt;, hors du mur.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -16660,10 +16660,10 @@
           <t>narrateur|Le jaune rejoint la grille, tout sec.
 copine|On a trouvé, Aniss.
 papa|Le vent n'a pas glissé.
-narrateur|Le porche a failli manger le vent.
+narrateur|Le caillou a failli trop peser.
 maman|Entrez, le seuil est sec.
 narrateur|Le caillou reste tiède, contre le barreau.
-narrateur|Un rai rouge s'allonge sur le bitume, puis s'arrête.
+narrateur|La pierre reste tiède, dans la paume.
 narrateur|Le vent pousse la goutte de cire rouge, hors du mur.</t>
         </is>
       </c>
@@ -16696,17 +16696,17 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Mila. Aniss pointe la marche, du doigt. Mila attend, puis ouvre les mains. Le caillou cale le papier sur la marche. Le courant du seuil pousse, tout net. Je le tiens. La goutte de cire rouge prend l'air, sur la marche. Le caillou attend, contre le papier. Le porche garde son ombre, plus loin. Tes mains ont guidé le moulin. Il tourne.</t>
+          <t>Mila. Aniss pointe la marche, du doigt. Mila attend, puis ouvre les mains. Le caillou cale le papier sur la marche. Le courant du seuil pousse, tout net. Je le tiens. La goutte de cire rouge prend l'air, sur la marche. Le caillou attend, contre le papier. Le porche garde son ombre, plus loin. Tes mains ont guidé le moulin. La marche.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila. Aniss pointe la &lt;emphasis level="moderate"&gt;marche&lt;/emphasis&gt;, du doigt. Mila attend, puis ouvre les mains. Le caillou cale le papier sur la marche. Le courant du seuil pousse, tout net. Je le tiens. La goutte de cire rouge prend l'air, sur la marche. Le caillou attend, contre le papier. Le porche garde son ombre, plus loin. Tes mains ont guidé le moulin. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila. Aniss pointe la &lt;emphasis level="moderate"&gt;marche&lt;/emphasis&gt;, du doigt. Mila attend, puis ouvre les mains. Le caillou cale le papier sur la marche. Le courant du seuil pousse, tout net. Je le tiens. La goutte de cire rouge prend l'air, sur la marche. Le caillou attend, contre le papier. Le porche garde son ombre, plus loin. Tes mains ont guidé le moulin. La marche.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Mila. Aniss pointe la &lt;emphasis&gt;marche&lt;/emphasis&gt;, du doigt. Mila attend, puis ouvre les mains. Le caillou cale le papier sur la marche. Le courant du seuil pousse, tout net. Je le tiens. La goutte de cire rouge prend l'air, sur la marche. Le caillou attend, contre le papier. Le porche garde son ombre, plus loin. Tes mains ont guidé le moulin. Il tourne. [pause]</t>
+          <t>Mila. Aniss pointe la &lt;emphasis&gt;marche&lt;/emphasis&gt;, du doigt. Mila attend, puis ouvre les mains. Le caillou cale le papier sur la marche. Le courant du seuil pousse, tout net. Je le tiens. La goutte de cire rouge prend l'air, sur la marche. Le caillou attend, contre le papier. Le porche garde son ombre, plus loin. Tes mains ont guidé le moulin. La marche. [pause]</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -16850,7 +16850,7 @@
 narrateur|Le caillou attend, contre le papier.
 maman|Le porche garde son ombre, plus loin.
 papa|Tes mains ont guidé le moulin.
-enfant-m|Il tourne.</t>
+enfant-m|La marche.</t>
         </is>
       </c>
       <c r="AX84" t="inlineStr">
@@ -16882,17 +16882,17 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Les mains de Mila laissent le jaune au fer. On l'a tenu, tous les deux. Le porche est resté à sa place. Le porche a failli manger le vent. Essuie tes chaussures, Aniss. Le caillou reste tiède, contre le barreau. Au muret, ça sent la cire, tiède. Deux pieds s'arrêtent, la goutte de cire rouge au milieu.</t>
+          <t>Les mains de Mila laissent le jaune au fer. On l'a tenu, tous les deux. Le porche est resté à sa place. Le caillou a failli trop peser. Essuie tes chaussures, Aniss. Le caillou reste tiède, contre le barreau. Un toc de fer s'éteint, tout près. Deux pieds s'arrêtent, la goutte de cire rouge au milieu.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les mains de Mila laissent le jaune au fer. On l'a tenu, tous les deux. Le porche est resté à sa place. Le porche a failli manger le vent. Essuie tes chaussures, Aniss. Le caillou reste tiède, contre le barreau. Au muret, ça sent la cire, tiède. Deux pieds s'arrêtent, la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; au milieu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les mains de Mila laissent le jaune au fer. On l'a tenu, tous les deux. Le porche est resté à sa place. Le caillou a failli trop peser. Essuie tes chaussures, Aniss. Le caillou reste tiède, contre le barreau. Un toc de fer s'éteint, tout près. Deux pieds s'arrêtent, la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; au milieu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les mains de Mila laissent le jaune au fer. On l'a tenu, tous les deux. Le porche est resté à sa place. Le porche a failli manger le vent. Essuie tes chaussures, Aniss. Le caillou reste tiède, contre le barreau. Au muret, ça sent la cire, tiède. Deux pieds s'arrêtent, la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; au milieu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les mains de Mila laissent le jaune au fer. On l'a tenu, tous les deux. Le porche est resté à sa place. Le caillou a failli trop peser. Essuie tes chaussures, Aniss. Le caillou reste tiède, contre le barreau. Un toc de fer s'éteint, tout près. Deux pieds s'arrêtent, la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; au milieu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr"/>
@@ -17033,10 +17033,10 @@
           <t>narrateur|Les mains de Mila laissent le jaune au fer.
 copine|On l'a tenu, tous les deux.
 papa|Le porche est resté à sa place.
-narrateur|Le porche a failli manger le vent.
+narrateur|Le caillou a failli trop peser.
 maman|Essuie tes chaussures, Aniss.
 narrateur|Le caillou reste tiède, contre le barreau.
-narrateur|Au muret, ça sent la cire, tiède.
+narrateur|Un toc de fer s'éteint, tout près.
 narrateur|Deux pieds s'arrêtent, la goutte de cire rouge au milieu.</t>
         </is>
       </c>
@@ -17069,17 +17069,17 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Le nœud, Aniss. Aniss pointe le crochet du porche, du doigt. Mila attend, puis suit le doigt. Le caillou tient derrière le nœud, tout droit. Le jaune se tient, hors du mur. Il évite le mur. La goutte de cire rouge veille derrière le nœud. Le caillou attend, contre le papier. Le nœud a montré la route. Vos pieds restent au sec, aussi. Il tourne.</t>
+          <t>Le nœud, Aniss. Aniss pointe le crochet du porche, du doigt. Mila attend, puis suit le doigt. Le caillou tient derrière le nœud, tout droit. Le jaune se tient, hors du mur. Il évite le mur. La goutte de cire rouge veille derrière le nœud. Le caillou attend, contre le papier. Le nœud a montré la route. Vos pieds restent au sec, aussi. Le nœud.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;nœud&lt;/emphasis&gt;, Aniss. Aniss pointe le crochet du porche, du doigt. Mila attend, puis suit le doigt. Le caillou tient derrière le nœud, tout droit. Le jaune se tient, hors du mur. Il évite le mur. La goutte de cire rouge veille derrière le nœud. Le caillou attend, contre le papier. Le nœud a montré la route. Vos pieds restent au sec, aussi. Il tourne.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;nœud&lt;/emphasis&gt;, Aniss. Aniss pointe le crochet du porche, du doigt. Mila attend, puis suit le doigt. Le caillou tient derrière le nœud, tout droit. Le jaune se tient, hors du mur. Il évite le mur. La goutte de cire rouge veille derrière le nœud. Le caillou attend, contre le papier. Le nœud a montré la route. Vos pieds restent au sec, aussi. Le nœud.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;nœud&lt;/emphasis&gt;, Aniss. Aniss pointe le crochet du porche, du doigt. Mila attend, puis suit le doigt. Le caillou tient derrière le nœud, tout droit. Le jaune se tient, hors du mur. Il évite le mur. La goutte de cire rouge veille derrière le nœud. Le caillou attend, contre le papier. Le nœud a montré la route. Vos pieds restent au sec, aussi. Il tourne. [pause]</t>
+          <t>Le &lt;emphasis&gt;nœud&lt;/emphasis&gt;, Aniss. Aniss pointe le crochet du porche, du doigt. Mila attend, puis suit le doigt. Le caillou tient derrière le nœud, tout droit. Le jaune se tient, hors du mur. Il évite le mur. La goutte de cire rouge veille derrière le nœud. Le caillou attend, contre le papier. Le nœud a montré la route. Vos pieds restent au sec, aussi. Le nœud. [pause]</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -17223,7 +17223,7 @@
 narrateur|Le caillou attend, contre le papier.
 papa|Le nœud a montré la route.
 maman|Vos pieds restent au sec, aussi.
-enfant-m|Il tourne.</t>
+enfant-m|Le nœud.</t>
         </is>
       </c>
       <c r="AX86" t="inlineStr">
@@ -17255,17 +17255,17 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Le jaune suit le nœud, jusqu'à la grille. L'ombre était douce. Le nœud a tenu, tout droit. Le porche a failli manger le vent. Le porche n'a plus rien à dire. Le caillou reste tiède, contre le barreau. Au loin, le bus se tait. Le papier tremble, la goutte de cire rouge se tait.</t>
+          <t>Le jaune suit le nœud, jusqu'à la grille. L'ombre était douce. Le nœud a tenu, tout droit. Le caillou a failli trop peser. Le porche n'a plus rien à dire. Le caillou reste tiède, contre le barreau. L'ombre du porche recule, un peu. Le papier tremble, la goutte de cire rouge se tait.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jaune suit le nœud, jusqu'à la grille. L'ombre était douce. Le nœud a tenu, tout droit. Le porche a failli manger le vent. Le porche n'a plus rien à dire. Le caillou reste tiède, contre le barreau. Au loin, le bus se tait. Le papier tremble, la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le jaune suit le nœud, jusqu'à la grille. L'ombre était douce. Le nœud a tenu, tout droit. Le caillou a failli trop peser. Le porche n'a plus rien à dire. Le caillou reste tiède, contre le barreau. L'ombre du porche recule, un peu. Le papier tremble, la &lt;emphasis level="moderate"&gt;goutte de cire rouge&lt;/emphasis&gt; se tait.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jaune suit le nœud, jusqu'à la grille. L'ombre était douce. Le nœud a tenu, tout droit. Le porche a failli manger le vent. Le porche n'a plus rien à dire. Le caillou reste tiède, contre le barreau. Au loin, le bus se tait. Le papier tremble, la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le jaune suit le nœud, jusqu'à la grille. L'ombre était douce. Le nœud a tenu, tout droit. Le caillou a failli trop peser. Le porche n'a plus rien à dire. Le caillou reste tiède, contre le barreau. L'ombre du porche recule, un peu. Le papier tremble, la &lt;emphasis&gt;goutte de cire rouge&lt;/emphasis&gt; se tait.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr"/>
@@ -17406,10 +17406,10 @@
           <t>narrateur|Le jaune suit le nœud, jusqu'à la grille.
 copine|L'ombre était douce.
 papa|Le nœud a tenu, tout droit.
-narrateur|Le porche a failli manger le vent.
+narrateur|Le caillou a failli trop peser.
 maman|Le porche n'a plus rien à dire.
 narrateur|Le caillou reste tiède, contre le barreau.
-narrateur|Au loin, le bus se tait.
+narrateur|L'ombre du porche recule, un peu.
 narrateur|Le papier tremble, la goutte de cire rouge se tait.</t>
         </is>
       </c>
@@ -17436,7 +17436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17500,6 +17500,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>